<commit_message>
T03: ghi chú khảo sát mảng B (Bệnh nhân & Lịch hẹn)
- Thêm docs/khao-sat/T03_KhaoSat_MangB.md: phạm vi, quy trình, thực thể,
  trạng thái lịch hẹn, BR-B01..B07, câu hỏi cần chốt
- Kế hoạch: T03 -> Hoàn thành 100%, chờ Đăng Khoa review
- Báo cáo tuần 1: ghi nhận T03 của Khôi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -23,7 +23,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kế hoạch'!$A$4:$L$59</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr fullCalcOnLoad="1" calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -2352,13 +2352,19 @@
       <c r="I7" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="J7" s="20" t="s">
-        <v>98</v>
+      <c r="J7" s="20" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
       </c>
       <c r="K7" s="21">
-        <v>0</v>
-      </c>
-      <c r="L7" s="22"/>
+        <v>1</v>
+      </c>
+      <c r="L7" s="22" t="inlineStr">
+        <is>
+          <t>docs/khao-sat/T03_KhaoSat_MangB.md – chờ Đăng Khoa review</t>
+        </is>
+      </c>
     </row>
     <row r="8" spans="1:12" ht="28" x14ac:dyDescent="0.2">
       <c r="A8" s="9" t="s">
@@ -4988,14 +4994,38 @@
         <v>357</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="20"/>
-      <c r="B6" s="31"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
+    <row r="6" spans="1:7" ht="84" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="20">
+        <v>1</v>
+      </c>
+      <c r="B6" s="31">
+        <v>46303</v>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>Khôi</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>T03: khảo sát quy trình đặt lịch, khám trực tiếp, tư vấn từ xa, chuyển chuyên khoa, thanh toán (Medpro, YouMed, BookingCare); đề xuất 6 thực thể, trạng thái lịch hẹn, BR-B01…B07 cho mảng B</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>T06: viết mục 1, 1.1. T08: chốt BR-B. T10: tổng hợp, nộp báo cáo v1</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>Cần nhóm chốt: (1) lưu giờ hẹn dạng khoảng thời gian + EXCLUDE hay bảng khung giờ; (2) BR-B03 có miễn tái khám không; (3) bỏ BAO_HIEM_Y_TE khỏi mảng B</t>
+        </is>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>https://github.com/khoiln218/telemedicine/blob/main/docs/khao-sat/T03_KhaoSat_MangB.md</t>
+        </is>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="20"/>

</xml_diff>

<commit_message>
T02: cấu trúc repo + README hướng dẫn cài đặt
- Thư mục erd/, sql/, app/; tài liệu môn học chuyển vào docs/de-bai/
- README: cấu trúc, cài PostgreSQL 16 + draw.io, tạo DB, thứ tự chạy SQL, quy ước
- .gitignore: file tạm Office/draw.io/Python, giáo trình và danh sách SV
- Kế hoạch: T02 -> Đang làm 80% (chờ 2 bạn cài theo README)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -2314,13 +2314,19 @@
       <c r="I6" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="J6" s="20" t="s">
-        <v>98</v>
+      <c r="J6" s="20" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
       </c>
       <c r="K6" s="21">
-        <v>0</v>
-      </c>
-      <c r="L6" s="22"/>
+        <v>0.8</v>
+      </c>
+      <c r="L6" s="22" t="inlineStr">
+        <is>
+          <t>Repo + cấu trúc thư mục + README xong; máy Khôi đã cài PG16 + draw.io. Chờ Hữu Khoa, Đăng Khoa cài theo README và báo lại</t>
+        </is>
+      </c>
     </row>
     <row r="7" spans="1:12" ht="28" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
@@ -5008,7 +5014,7 @@
       </c>
       <c r="D6" s="22" t="inlineStr">
         <is>
-          <t>T03: khảo sát quy trình đặt lịch, khám trực tiếp, tư vấn từ xa, chuyển chuyên khoa, thanh toán (Medpro, YouMed, BookingCare); đề xuất 6 thực thể, trạng thái lịch hẹn, BR-B01…B07 cho mảng B</t>
+          <t>T02: cấu trúc repo (docs, erd, sql, app), README cài PostgreSQL 16 + draw.io, .gitignore; gỡ giáo trình và danh sách SV khỏi repo public. T03: khảo sát quy trình đặt lịch, khám trực tiếp, tư vấn từ xa, chuyển chuyên khoa, thanh toán (Medpro, YouMed, BookingCare); đề xuất 6 thực thể, trạng thái lịch hẹn, BR-B01…B07 cho mảng B</t>
         </is>
       </c>
       <c r="E6" s="22" t="inlineStr">

</xml_diff>

<commit_message>
T08: quy tắc nghiệp vụ mảng B (BR-B01..B11)
- Thêm docs/br/T08_BR_MangB.md: bảng BR cho mục 1.2.2, cách kiểm chứng,
  liên kết MT, phụ thuộc mảng A
- Chốt: giờ hẹn dạng khoảng + EXCLUDE, tái khám miễn giấy chuyển
- Kế hoạch: T08 -> Hoàn thành 100%, chờ Hữu Khoa review

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -2554,13 +2554,19 @@
       <c r="I12" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="J12" s="20" t="s">
-        <v>98</v>
+      <c r="J12" s="20" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
       </c>
       <c r="K12" s="21">
-        <v>0</v>
-      </c>
-      <c r="L12" s="22"/>
+        <v>1</v>
+      </c>
+      <c r="L12" s="22" t="inlineStr">
+        <is>
+          <t>docs/br/T08_BR_MangB.md (BR-B01…B11) – chờ Hữu Khoa review, xác nhận phụ thuộc mảng A</t>
+        </is>
+      </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
@@ -5014,17 +5020,17 @@
       </c>
       <c r="D6" s="22" t="inlineStr">
         <is>
-          <t>T02: cấu trúc repo (docs, erd, sql, app), README cài PostgreSQL 16 + draw.io, .gitignore; gỡ giáo trình và danh sách SV khỏi repo public. T03: khảo sát quy trình đặt lịch, khám trực tiếp, tư vấn từ xa, chuyển chuyên khoa, thanh toán (Medpro, YouMed, BookingCare); đề xuất 6 thực thể, trạng thái lịch hẹn, BR-B01…B07 cho mảng B</t>
+          <t>T02: cấu trúc repo (docs, erd, sql, app), README cài PostgreSQL 16 + draw.io, .gitignore; gỡ giáo trình và danh sách SV khỏi repo public. T03: khảo sát quy trình đặt lịch, khám trực tiếp, tư vấn từ xa, chuyển chuyên khoa, thanh toán (Medpro, YouMed, BookingCare); đề xuất 6 thực thể, trạng thái lịch hẹn, BR-B01…B07 cho mảng B. T08: viết BR-B01…B11 kèm cơ chế và cách kiểm chứng, chốt 2 câu hỏi mở của T03; chạy thử EXCLUDE cho BR-B02 trên PG16</t>
         </is>
       </c>
       <c r="E6" s="22" t="inlineStr">
         <is>
-          <t>T06: viết mục 1, 1.1. T08: chốt BR-B. T10: tổng hợp, nộp báo cáo v1</t>
+          <t>T06: viết mục 1, 1.1. T10: tổng hợp mục 1.2, nộp báo cáo v1</t>
         </is>
       </c>
       <c r="F6" s="22" t="inlineStr">
         <is>
-          <t>Cần nhóm chốt: (1) lưu giờ hẹn dạng khoảng thời gian + EXCLUDE hay bảng khung giờ; (2) BR-B03 có miễn tái khám không; (3) bỏ BAO_HIEM_Y_TE khỏi mảng B</t>
+          <t>Cần nhóm chốt: Hữu Khoa xác nhận phương án ánh xạ lớp bác sĩ đa khoa (ảnh hưởng BR-B09); nhóm đồng ý bỏ BAO_HIEM_Y_TE khỏi mảng B</t>
         </is>
       </c>
       <c r="G6" s="22" t="inlineStr">

</xml_diff>

<commit_message>
T06: báo cáo mục 1 và 1.1
- Mục 1: bối cảnh, quy mô giả định, vấn đề hiện tại; bảng phạm vi,
  tác nhân, thuật ngữ (thay chữ gợi ý xám bằng nội dung thật)
- Mục 1.1: MT-01..MT-07 kèm tiêu chí kiểm chứng và liên kết BR/Q/TC
- Kế hoạch: T06 -> Hoàn thành 100%; Viết báo cáo: mục 1, 1.1 hoàn thành
- Báo cáo tuần 1 (Khôi): viết lại gọn theo từng việc T02, T03, T08, T06,
  vướng mắc theo người, link sản phẩm
- Kế hoạch: việc "Hoàn thành" tự gạch ngang cột Công việc, chữ xám ở
  A–E, G–I (định dạng có điều kiện)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khoile/Documents/PTIT/HK5/CSDL/telemedicine/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F88FD1E-811B-A04B-A405-3BB62743EB9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F01E9CA-2B7C-5143-AC4B-D6047880E334}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1180" yWindow="660" windowWidth="29060" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kế hoạch'!$A$4:$L$59</definedName>
   </definedNames>
-  <calcPr fullCalcOnLoad="1" calcId="191029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="379">
   <si>
     <t>Kế hoạch đồ án – Nhóm G5 – Đề tài #5: Cổng thông tin phòng khám &amp; y tế từ xa (Telemedicine)</t>
   </si>
@@ -1205,6 +1205,39 @@
   </si>
   <si>
     <t>Ghi chú: việc của 'Cả nhóm' tính riêng; dùng bảng này cùng sheet 'Báo cáo tuần' làm căn cứ cho đánh giá chéo (15% điểm cá nhân).</t>
+  </si>
+  <si>
+    <t>Repo + cấu trúc thư mục + README xong; máy Khôi đã cài PG16 + draw.io. Chờ Hữu Khoa, Đăng Khoa cài theo README và báo lại</t>
+  </si>
+  <si>
+    <t>docs/khao-sat/T03_KhaoSat_MangB.md – chờ Đăng Khoa review</t>
+  </si>
+  <si>
+    <t>docs/br/T08_BR_MangB.md (BR-B01…B11) – chờ Hữu Khoa review, xác nhận phụ thuộc mảng A</t>
+  </si>
+  <si>
+    <t>Đã điền mục 1, 1.1 vào docs/INT1313_TX_G5_DeTai05_Telemedicine_v0.docx – chờ Hữu Khoa review</t>
+  </si>
+  <si>
+    <t>T02: cấu trúc repo, README cài PostgreSQL 16 + draw.io, gỡ file nhạy cảm khỏi repo public
+T03: khảo sát mảng B (Medpro, YouMed, BookingCare), đề xuất 6 thực thể
+T08: BR-B01…B11 kèm cơ chế và cách kiểm chứng; chạy thử EXCLUDE chống trùng lịch trên PG16
+T06: báo cáo mục 1 và 1.1 (MT-01…07)</t>
+  </si>
+  <si>
+    <t>T10: gộp mục 1.2 (BR mảng A, C), review chéo, nộp báo cáo v1</t>
+  </si>
+  <si>
+    <t>Hữu Khoa: chốt phương án ánh xạ lớp bác sĩ đa khoa (ảnh hưởng BR-B09)
+Cả nhóm: đồng ý bỏ BAO_HIEM_Y_TE khỏi mảng B
+Đăng Khoa: giữ số hiệu BR-C01…C05 vì MT-04, MT-05 đang tham chiếu</t>
+  </si>
+  <si>
+    <t>github.com/khoiln218/telemedicine
+README.md
+docs/khao-sat/T03_KhaoSat_MangB.md
+docs/br/T08_BR_MangB.md
+docs/…_v0.docx (mục 1, 1.1)</t>
   </si>
 </sst>
 </file>
@@ -1476,7 +1509,28 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="7">
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF808080"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike/>
+        <color rgb="FF808080"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2284,7 +2338,7 @@
       </c>
       <c r="L5" s="22"/>
     </row>
-    <row r="6" spans="1:12" ht="28" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" ht="70" x14ac:dyDescent="0.2">
       <c r="A6" s="9" t="s">
         <v>99</v>
       </c>
@@ -2314,21 +2368,17 @@
       <c r="I6" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="J6" s="20" t="inlineStr">
-        <is>
-          <t>Đang làm</t>
-        </is>
+      <c r="J6" s="20" t="s">
+        <v>362</v>
       </c>
       <c r="K6" s="21">
         <v>0.8</v>
       </c>
-      <c r="L6" s="22" t="inlineStr">
-        <is>
-          <t>Repo + cấu trúc thư mục + README xong; máy Khôi đã cài PG16 + draw.io. Chờ Hữu Khoa, Đăng Khoa cài theo README và báo lại</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="28" x14ac:dyDescent="0.2">
+      <c r="L6" s="22" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="42" x14ac:dyDescent="0.2">
       <c r="A7" s="9" t="s">
         <v>102</v>
       </c>
@@ -2358,18 +2408,14 @@
       <c r="I7" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="J7" s="20" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
+      <c r="J7" s="20" t="s">
+        <v>361</v>
       </c>
       <c r="K7" s="21">
         <v>1</v>
       </c>
-      <c r="L7" s="22" t="inlineStr">
-        <is>
-          <t>docs/khao-sat/T03_KhaoSat_MangB.md – chờ Đăng Khoa review</t>
-        </is>
+      <c r="L7" s="22" t="s">
+        <v>372</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="28" x14ac:dyDescent="0.2">
@@ -2448,7 +2494,7 @@
       </c>
       <c r="L9" s="22"/>
     </row>
-    <row r="10" spans="1:12" ht="28" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" ht="56" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
         <v>111</v>
       </c>
@@ -2479,12 +2525,14 @@
         <v>113</v>
       </c>
       <c r="J10" s="20" t="s">
-        <v>98</v>
+        <v>361</v>
       </c>
       <c r="K10" s="21">
-        <v>0</v>
-      </c>
-      <c r="L10" s="22"/>
+        <v>1</v>
+      </c>
+      <c r="L10" s="22" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="11" spans="1:12" ht="28" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
@@ -2524,7 +2572,7 @@
       </c>
       <c r="L11" s="22"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="56" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
         <v>117</v>
       </c>
@@ -2554,18 +2602,14 @@
       <c r="I12" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="J12" s="20" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
+      <c r="J12" s="20" t="s">
+        <v>361</v>
       </c>
       <c r="K12" s="21">
         <v>1</v>
       </c>
-      <c r="L12" s="22" t="inlineStr">
-        <is>
-          <t>docs/br/T08_BR_MangB.md (BR-B01…B11) – chờ Hữu Khoa review, xác nhận phụ thuộc mảng A</t>
-        </is>
+      <c r="L12" s="22" t="s">
+        <v>373</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
@@ -4357,14 +4401,29 @@
   </sheetData>
   <autoFilter ref="A4:L59" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <conditionalFormatting sqref="J5:J109">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
       <formula>"Hoàn thành"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
       <formula>"Đang làm"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
       <formula>"Trễ hạn"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F5:F109">
+    <cfRule type="expression" dxfId="3" priority="5" stopIfTrue="1">
+      <formula>$J5="Hoàn thành"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:E109">
+    <cfRule type="expression" dxfId="2" priority="6" stopIfTrue="1">
+      <formula>$J5="Hoàn thành"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G5:I109">
+    <cfRule type="expression" dxfId="1" priority="7" stopIfTrue="1">
+      <formula>$J5="Hoàn thành"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
@@ -4602,7 +4661,7 @@
         <v>12</v>
       </c>
       <c r="G5" s="20" t="s">
-        <v>98</v>
+        <v>361</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -4625,7 +4684,7 @@
         <v>2</v>
       </c>
       <c r="G6" s="20" t="s">
-        <v>98</v>
+        <v>361</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -5006,37 +5065,27 @@
         <v>357</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="84" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="98" x14ac:dyDescent="0.2">
       <c r="A6" s="20">
         <v>1</v>
       </c>
       <c r="B6" s="31">
         <v>46303</v>
       </c>
-      <c r="C6" s="20" t="inlineStr">
-        <is>
-          <t>Khôi</t>
-        </is>
-      </c>
-      <c r="D6" s="22" t="inlineStr">
-        <is>
-          <t>T02: cấu trúc repo (docs, erd, sql, app), README cài PostgreSQL 16 + draw.io, .gitignore; gỡ giáo trình và danh sách SV khỏi repo public. T03: khảo sát quy trình đặt lịch, khám trực tiếp, tư vấn từ xa, chuyển chuyên khoa, thanh toán (Medpro, YouMed, BookingCare); đề xuất 6 thực thể, trạng thái lịch hẹn, BR-B01…B07 cho mảng B. T08: viết BR-B01…B11 kèm cơ chế và cách kiểm chứng, chốt 2 câu hỏi mở của T03; chạy thử EXCLUDE cho BR-B02 trên PG16</t>
-        </is>
-      </c>
-      <c r="E6" s="22" t="inlineStr">
-        <is>
-          <t>T06: viết mục 1, 1.1. T10: tổng hợp mục 1.2, nộp báo cáo v1</t>
-        </is>
-      </c>
-      <c r="F6" s="22" t="inlineStr">
-        <is>
-          <t>Cần nhóm chốt: Hữu Khoa xác nhận phương án ánh xạ lớp bác sĩ đa khoa (ảnh hưởng BR-B09); nhóm đồng ý bỏ BAO_HIEM_Y_TE khỏi mảng B</t>
-        </is>
-      </c>
-      <c r="G6" s="22" t="inlineStr">
-        <is>
-          <t>https://github.com/khoiln218/telemedicine/blob/main/docs/khao-sat/T03_KhaoSat_MangB.md</t>
-        </is>
+      <c r="C6" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>375</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>376</v>
+      </c>
+      <c r="F6" s="22" t="s">
+        <v>377</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>378</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -5901,11 +5950,11 @@
       </c>
       <c r="C5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Hoàn thành")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Đang làm")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Trễ hạn")</f>
@@ -5913,11 +5962,11 @@
       </c>
       <c r="F5" s="34">
         <f>IFERROR(C5/B5,0)</f>
-        <v>0</v>
+        <v>0.15789473684210525</v>
       </c>
       <c r="G5" s="34">
         <f>IFERROR(AVERAGEIF('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0</v>
+        <v>0.19999999999999998</v>
       </c>
       <c r="H5" s="7">
         <f>COUNTIF('Kế hoạch'!$H$5:$H$109,A5)</f>
@@ -6033,11 +6082,11 @@
       </c>
       <c r="C9" s="35">
         <f>SUM(C5:C8)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D9" s="35">
         <f>SUM(D5:D8)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="35">
         <f>SUM(E5:E8)</f>
@@ -6045,11 +6094,11 @@
       </c>
       <c r="F9" s="36">
         <f>IFERROR(C9/B9,0)</f>
-        <v>0</v>
+        <v>5.4545454545454543E-2</v>
       </c>
       <c r="G9" s="36">
         <f>IFERROR(AVERAGE('Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0</v>
+        <v>6.9090909090909092E-2</v>
       </c>
       <c r="H9" s="35">
         <f>SUM(H5:H8)</f>
@@ -6085,11 +6134,11 @@
       </c>
       <c r="C14" s="9">
         <f>COUNTIFS('Kế hoạch'!$E$5:$E$109,A14,'Kế hoạch'!$J$5:$J$109,"Hoàn thành")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D14" s="37">
         <f>IFERROR(C14/B14,0)</f>
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
T07 T09: cập nhật kế hoạch sau review mảng A, C
- T05: Hoàn thành, chờ Hữu Khoa review
- T07: Đang làm 70%, ghi các điểm cần sửa của BR_MangA (giữ số hiệu BR-A01…A04 như v0)
- T09: Đang làm 90%, ghi các điểm cần sửa và đề xuất chốt của BR mảng C
- T10: ghi chú khi gộp v0

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -23,7 +23,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kế hoạch'!$A$4:$L$59</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="383">
   <si>
     <t>Kế hoạch đồ án – Nhóm G5 – Đề tài #5: Cổng thông tin phòng khám &amp; y tế từ xa (Telemedicine)</t>
   </si>
@@ -1238,6 +1238,18 @@
 docs/khao-sat/T03_KhaoSat_MangB.md
 docs/br/T08_BR_MangB.md
 docs/…_v0.docx (mục 1, 1.1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/khao-sat/T05_KhaoSat_MangC.md – chờ Hữu Khoa review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/br/T09_BR_MangC.md – Khôi review 14/10, cần sửa: (1) LAN_KHAM bỏ ma_bn, ma_bac_si; DON_THUOC bỏ ma_bac_si_ke (3NF); (2) BR-C02 dẫn BR-B05; (3) định nghĩa "dị ứng còn hiệu lực"; (4) BR-C03 dựa BR-C05 để chặn xóa chẩn đoán. Thêm tên trigger theo v0, TC-06, mục phụ thuộc A/B. Đề xuất chốt: 1 hồ sơ/BN; lần khám chỉ tạo khi lịch HOAN_THANH; liều lưu văn bản; chặn DELETE 5 bảng bệnh án; chỉ kiểm tra dị ứng khi kê.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khi gộp v0: BR_MangA phải giữ số hiệu BR-A01…A04 như v0 (MT-01, TC-03, 4.1.4 đang dùng); thống nhất kiểu mã test TC-xx / TC-A01-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/br/BR_MangA.md – Khôi review 14/10, cần sửa: (1) giữ BR-A01…A04 như v0 (MT-01, TC-03, 4.1.4 đang dùng), quy tắc mới đánh từ A05; (2) bỏ các quy tắc chỉ là PK/FK, đưa sang từ điển dữ liệu; (3) định nghĩa cụ thể: ca còn hiệu lực = trạng thái khác HUY, chứng chỉ còn hạn = ngày hết hạn ≥ ngày kết thúc ca; (4) A13 → không sửa/hủy ca nếu làm lịch hẹn còn hiệu lực rơi ra ngoài ca; (5) bỏ A12 (lịch hẹn không có cột chuyên khoa); (6) đề xuất mỗi BS chuyên khoa thuộc đúng 1 chuyên khoa; ca chồng giờ dùng EXCLUDE như BR-B02. Đổi tên T07_BR_MangA.md, gọn theo dạng T08. T04 (khảo sát mảng A) chưa có.</t>
   </si>
 </sst>
 </file>
@@ -2456,7 +2468,7 @@
       </c>
       <c r="L8" s="22"/>
     </row>
-    <row r="9" spans="1:12" ht="28" x14ac:dyDescent="0.2">
+    <row r="9" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="9" t="s">
         <v>108</v>
       </c>
@@ -2487,12 +2499,14 @@
         <v>110</v>
       </c>
       <c r="J9" s="20" t="s">
-        <v>98</v>
+        <v>361</v>
       </c>
       <c r="K9" s="21">
-        <v>0</v>
-      </c>
-      <c r="L9" s="22"/>
+        <v>1</v>
+      </c>
+      <c r="L9" s="22" t="s">
+        <v>379</v>
+      </c>
     </row>
     <row r="10" spans="1:12" ht="56" x14ac:dyDescent="0.2">
       <c r="A10" s="9" t="s">
@@ -2534,7 +2548,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="28" x14ac:dyDescent="0.2">
+    <row r="11" ht="330" customHeight="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="9" t="s">
         <v>114</v>
       </c>
@@ -2565,12 +2579,14 @@
         <v>116</v>
       </c>
       <c r="J11" s="20" t="s">
-        <v>98</v>
+        <v>362</v>
       </c>
       <c r="K11" s="21">
-        <v>0</v>
-      </c>
-      <c r="L11" s="22"/>
+        <v>0.7</v>
+      </c>
+      <c r="L11" s="22" t="s">
+        <v>382</v>
+      </c>
     </row>
     <row r="12" spans="1:12" ht="56" x14ac:dyDescent="0.2">
       <c r="A12" s="9" t="s">
@@ -2612,7 +2628,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" ht="230" customHeight="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
         <v>120</v>
       </c>
@@ -2643,14 +2659,16 @@
         <v>122</v>
       </c>
       <c r="J13" s="20" t="s">
-        <v>98</v>
+        <v>362</v>
       </c>
       <c r="K13" s="21">
-        <v>0</v>
-      </c>
-      <c r="L13" s="22"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+        <v>0.9</v>
+      </c>
+      <c r="L13" s="22" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="14" ht="80" customHeight="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
         <v>123</v>
       </c>
@@ -2686,7 +2704,9 @@
       <c r="K14" s="21">
         <v>0</v>
       </c>
-      <c r="L14" s="22"/>
+      <c r="L14" s="22" t="s">
+        <v>381</v>
+      </c>
     </row>
     <row r="15" spans="1:12" ht="28" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">

</xml_diff>

<commit_message>
T10: gộp mục 1.2 vào báo cáo v1
- Đổi tên báo cáo sang _v1.docx, cập nhật dòng phiên bản
- Mục 1.2: BR-A01…A08 (gộp theo review, giữ A01–A04 như v0), BR-B01…B11, BR-C01…C05; 1.2.4 ràng buộc chung
- Kế hoạch: T10 Đang làm 80%, trạng thái mục 1.1/1.2, báo cáo tuần 2 của Khôi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="387">
   <si>
     <t>Kế hoạch đồ án – Nhóm G5 – Đề tài #5: Cổng thông tin phòng khám &amp; y tế từ xa (Telemedicine)</t>
   </si>
@@ -1246,10 +1246,25 @@
     <t xml:space="preserve">docs/br/T09_BR_MangC.md – Khôi review 14/10, cần sửa: (1) LAN_KHAM bỏ ma_bn, ma_bac_si; DON_THUOC bỏ ma_bac_si_ke (3NF); (2) BR-C02 dẫn BR-B05; (3) định nghĩa "dị ứng còn hiệu lực"; (4) BR-C03 dựa BR-C05 để chặn xóa chẩn đoán. Thêm tên trigger theo v0, TC-06, mục phụ thuộc A/B. Đề xuất chốt: 1 hồ sơ/BN; lần khám chỉ tạo khi lịch HOAN_THANH; liều lưu văn bản; chặn DELETE 5 bảng bệnh án; chỉ kiểm tra dị ứng khi kê.</t>
   </si>
   <si>
-    <t xml:space="preserve">Khi gộp v0: BR_MangA phải giữ số hiệu BR-A01…A04 như v0 (MT-01, TC-03, 4.1.4 đang dùng); thống nhất kiểu mã test TC-xx / TC-A01-01</t>
+    <t xml:space="preserve">docs/INT1313_TX_G5_DeTai05_Telemedicine_v1.docx: đã gộp mục 1.2 (BR-A01…A08 theo review, giữ A01–A04 như v0; BR-B01…B11; BR-C01…C05) và 1.2.4. Còn: Hữu Khoa, Đăng Khoa xác nhận 1.2.1/1.2.3; Hữu Khoa review mảng B; điền ngày nộp; nộp v1 + báo cáo tiến độ. Lưu ý 4.1.4: trg_lich_hen_hop_le ghi BR-B01, B02 nhưng theo T08 là BR-B01, B03 (B02 dùng EXCLUDE).</t>
   </si>
   <si>
     <t xml:space="preserve">docs/br/BR_MangA.md – Khôi review 14/10, cần sửa: (1) giữ BR-A01…A04 như v0 (MT-01, TC-03, 4.1.4 đang dùng), quy tắc mới đánh từ A05; (2) bỏ các quy tắc chỉ là PK/FK, đưa sang từ điển dữ liệu; (3) định nghĩa cụ thể: ca còn hiệu lực = trạng thái khác HUY, chứng chỉ còn hạn = ngày hết hạn ≥ ngày kết thúc ca; (4) A13 → không sửa/hủy ca nếu làm lịch hẹn còn hiệu lực rơi ra ngoài ca; (5) bỏ A12 (lịch hẹn không có cột chuyên khoa); (6) đề xuất mỗi BS chuyên khoa thuộc đúng 1 chuyên khoa; ca chồng giờ dùng EXCLUDE như BR-B02. Đổi tên T07_BR_MangA.md, gọn theo dạng T08. T04 (khảo sát mảng A) chưa có.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T10: review chéo BR mảng A (BR_MangA.md) và C (T09), ghi điểm cần sửa vào kế hoạch; gộp mục 1.2 + 1.2.4 vào báo cáo v1 (docx đổi tên _v1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T10: chốt 1.2 với Hữu Khoa, Đăng Khoa, nộp v1 + báo cáo tiến độ. T12: vẽ ER/EER mảng B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hữu Khoa: xác nhận BR-A01…A08 theo review (giữ số hiệu v0), review BR mảng B
+Đăng Khoa: sửa T09 theo review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/INT1313_TX_G5_DeTai05_Telemedicine_v1.docx
+docs/KeHoach_G5_Telemedicine.xlsx
+nhánh member/Khoi</t>
   </si>
 </sst>
 </file>
@@ -2668,7 +2683,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="14" ht="80" customHeight="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" ht="200" customHeight="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="9" t="s">
         <v>123</v>
       </c>
@@ -2699,10 +2714,10 @@
         <v>125</v>
       </c>
       <c r="J14" s="20" t="s">
-        <v>98</v>
+        <v>362</v>
       </c>
       <c r="K14" s="21">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="L14" s="22" t="s">
         <v>381</v>
@@ -4727,7 +4742,7 @@
         <v>2</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>98</v>
+        <v>361</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -4750,7 +4765,7 @@
         <v>2</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>98</v>
+        <v>362</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -5108,14 +5123,28 @@
         <v>378</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="20"/>
-      <c r="B7" s="31"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
+    <row r="7" spans="1:7" ht="98" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="20">
+        <v>2</v>
+      </c>
+      <c r="B7" s="31">
+        <v>46309</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>383</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>384</v>
+      </c>
+      <c r="F7" s="22" t="s">
+        <v>385</v>
+      </c>
+      <c r="G7" s="22" t="s">
+        <v>386</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="20"/>

</xml_diff>

<commit_message>
T24: FD và khóa ứng viên mảng B; cập nhật kế hoạch T20, T24
FD (phủ tối thiểu), FD đã xét và loại kèm lý do, khóa ứng viên cho
BENH_NHAN, GIAY_CHUYEN_KHOA, LICH_HEN, TAI_KHOAN; nêu điểm cần chốt ở
T27/T30. README thêm thư mục docs/6_chuan-hoa. Kế hoạch: T20, T24 hoàn
thành, báo cáo tuần 4, mục 2.2 đang làm.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11023"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khoile/Documents/PTIT/HK5/CSDL/telemedicine/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3348BEEE-16D4-854B-A642-9A911A355645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2449E06F-5546-5647-AB5C-A083A0E33009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1180" yWindow="660" windowWidth="29060" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1200" yWindow="660" windowWidth="29040" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tổng quan" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="405">
   <si>
     <t>Kế hoạch công việc theo tuần</t>
   </si>
@@ -1314,6 +1314,28 @@
   </si>
   <si>
     <t>Ghi chú: việc của 'Cả nhóm' tính riêng; dùng bảng này cùng sheet 'Báo cáo tuần' làm căn cứ cho đánh giá chéo (15% điểm cá nhân).</t>
+  </si>
+  <si>
+    <t>docs/5_anh-xa/T20_AnhXa_MangB.md – 4 bảng BENH_NHAN, GIAY_CHUYEN_KHOA, LICH_HEN, TAI_KHOAN; PK/FK theo Elmasri bước 1–8, LICH_HEN chọn 8C (27/10); chờ Hữu Khoa review, xác nhận 8A cho BAC_SI (T19)</t>
+  </si>
+  <si>
+    <t>docs/6_chuan-hoa/T24_FD_MangB.md – FD (phủ tối thiểu), FD đã loại kèm lý do, khóa ứng viên 4 bảng; BENH_NHAN có 2 khóa {ma_bn}, {sdt} (27/10); chờ Đăng Khoa review</t>
+  </si>
+  <si>
+    <t>T20: ánh xạ mảng B sang lược đồ quan hệ (Elmasri bước 1–8): 4 bảng, PK/FK, UNIQUE; phân lớp LICH_HEN chọn 8C; truy vết ERD → lược đồ, quy tắc còn lại cho cài đặt
+T24: FD và khóa ứng viên 4 bảng mảng B, ghi FD đã xét và loại; nêu 2 điểm cho T27/T30 (FD có điều kiện trên cột UNIQUE cho phép NULL; TAI_KHOAN.vai_tro trùng NHAN_VIEN.loai_nv)</t>
+  </si>
+  <si>
+    <t>T27: chứng minh 3NF/BCNF mảng B. T21: review ánh xạ mảng C</t>
+  </si>
+  <si>
+    <t>Hữu Khoa: chốt phương án ánh xạ BAC_SI (8A hay 8C) ở T19 – ảnh hưởng FK ma_bac_si_lap → BAC_SI_DA_KHOA; review T20
+Đăng Khoa: review T24; chốt cách trình bày FD có điều kiện ở T22</t>
+  </si>
+  <si>
+    <t>docs/5_anh-xa/T20_AnhXa_MangB.md
+commit 78857c7, nhánh Khoi
+docs/6_chuan-hoa/T24_FD_MangB.md</t>
   </si>
 </sst>
 </file>
@@ -3125,7 +3147,7 @@
       </c>
       <c r="L23" s="22"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12" ht="126" x14ac:dyDescent="0.2">
       <c r="A24" s="13" t="s">
         <v>97</v>
       </c>
@@ -3156,12 +3178,14 @@
         <v>99</v>
       </c>
       <c r="J24" s="20" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="K24" s="21">
-        <v>0</v>
-      </c>
-      <c r="L24" s="22"/>
+        <v>1</v>
+      </c>
+      <c r="L24" s="22" t="s">
+        <v>399</v>
+      </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="13" t="s">
@@ -3277,7 +3301,7 @@
       </c>
       <c r="L27" s="22"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" ht="98" x14ac:dyDescent="0.2">
       <c r="A28" s="13" t="s">
         <v>109</v>
       </c>
@@ -3308,12 +3332,14 @@
         <v>111</v>
       </c>
       <c r="J28" s="20" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="K28" s="21">
-        <v>0</v>
-      </c>
-      <c r="L28" s="22"/>
+        <v>1</v>
+      </c>
+      <c r="L28" s="22" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="13" t="s">
@@ -4894,7 +4920,7 @@
         <v>8</v>
       </c>
       <c r="G11" s="20" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -5229,14 +5255,28 @@
         <v>387</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="20"/>
-      <c r="B9" s="31"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
+    <row r="9" spans="1:7" ht="112" x14ac:dyDescent="0.2">
+      <c r="A9" s="20">
+        <v>4</v>
+      </c>
+      <c r="B9" s="31">
+        <v>46322</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>401</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>402</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>403</v>
+      </c>
+      <c r="G9" s="22" t="s">
+        <v>404</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="20"/>
@@ -6073,7 +6113,7 @@
       </c>
       <c r="C5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Hoàn thành")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Đang làm")</f>
@@ -6085,11 +6125,11 @@
       </c>
       <c r="F5" s="34">
         <f>IFERROR(C5/B5,0)</f>
-        <v>0.26315789473684209</v>
+        <v>0.36842105263157893</v>
       </c>
       <c r="G5" s="34">
         <f>IFERROR(AVERAGEIF('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.35263157894736841</v>
+        <v>0.45789473684210524</v>
       </c>
       <c r="H5" s="7">
         <f>COUNTIF('Kế hoạch'!$H$5:$H$109,A5)</f>
@@ -6205,7 +6245,7 @@
       </c>
       <c r="C9" s="35">
         <f>SUM(C5:C8)</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D9" s="35">
         <f>SUM(D5:D8)</f>
@@ -6217,11 +6257,11 @@
       </c>
       <c r="F9" s="36">
         <f>IFERROR(C9/B9,0)</f>
-        <v>0.25454545454545452</v>
+        <v>0.29090909090909089</v>
       </c>
       <c r="G9" s="36">
         <f>IFERROR(AVERAGE('Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.28545454545454546</v>
+        <v>0.32181818181818189</v>
       </c>
       <c r="H9" s="35">
         <f>SUM(H5:H8)</f>
@@ -6291,11 +6331,11 @@
       </c>
       <c r="C16" s="13">
         <f>COUNTIFS('Kế hoạch'!$E$5:$E$109,A16,'Kế hoạch'!$J$5:$J$109,"Hoàn thành")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D16" s="39">
         <f>IFERROR(C16/B16,0)</f>
-        <v>0</v>
+        <v>0.14285714285714285</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
T27: chứng minh chuẩn hóa mảng B (BCNF, không tách bảng); cập nhật kế hoạch
1NF → BCNF cho BENH_NHAN, GIAY_CHUYEN_KHOA, LICH_HEN, TAI_KHOAN; lập luận
riêng cho FD có điều kiện trên cột UNIQUE cho phép NULL; ghi các thiết kế
đã tránh vi phạm 3NF; TAI_KHOAN.vai_tro trùng loai_nv chuyển T30.
Kế hoạch: T27 hoàn thành, mục 2.3 đang làm, báo cáo tuần 4.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khoile/Documents/PTIT/HK5/CSDL/telemedicine/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2449E06F-5546-5647-AB5C-A083A0E33009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F582DAB-94D2-584F-B51A-17E84C7944A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1200" yWindow="660" windowWidth="29040" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="406">
   <si>
     <t>Kế hoạch công việc theo tuần</t>
   </si>
@@ -1322,20 +1322,26 @@
     <t>docs/6_chuan-hoa/T24_FD_MangB.md – FD (phủ tối thiểu), FD đã loại kèm lý do, khóa ứng viên 4 bảng; BENH_NHAN có 2 khóa {ma_bn}, {sdt} (27/10); chờ Đăng Khoa review</t>
   </si>
   <si>
+    <t>docs/6_chuan-hoa/T27_ChuanHoa_MangB.md – 4 bảng đạt BCNF, không tách; lập luận riêng cho FD có điều kiện (cột UNIQUE cho phép NULL); vai_tro trùng loai_nv chuyển T30 (27/10); chờ Đăng Khoa review</t>
+  </si>
+  <si>
     <t>T20: ánh xạ mảng B sang lược đồ quan hệ (Elmasri bước 1–8): 4 bảng, PK/FK, UNIQUE; phân lớp LICH_HEN chọn 8C; truy vết ERD → lược đồ, quy tắc còn lại cho cài đặt
-T24: FD và khóa ứng viên 4 bảng mảng B, ghi FD đã xét và loại; nêu 2 điểm cho T27/T30 (FD có điều kiện trên cột UNIQUE cho phép NULL; TAI_KHOAN.vai_tro trùng NHAN_VIEN.loai_nv)</t>
-  </si>
-  <si>
-    <t>T27: chứng minh 3NF/BCNF mảng B. T21: review ánh xạ mảng C</t>
+T24: FD và khóa ứng viên 4 bảng mảng B, ghi FD đã xét và loại; nêu 2 điểm cho T27/T30 (FD có điều kiện trên cột UNIQUE cho phép NULL; TAI_KHOAN.vai_tro trùng NHAN_VIEN.loai_nv)
+T27: chứng minh 1NF → BCNF 4 bảng mảng B, không phải tách; ghi các thiết kế đã tránh vi phạm 3NF</t>
+  </si>
+  <si>
+    <t>T21: review ánh xạ mảng C. T29: điền từ điển dữ liệu bảng mảng B</t>
   </si>
   <si>
     <t>Hữu Khoa: chốt phương án ánh xạ BAC_SI (8A hay 8C) ở T19 – ảnh hưởng FK ma_bac_si_lap → BAC_SI_DA_KHOA; review T20
-Đăng Khoa: review T24; chốt cách trình bày FD có điều kiện ở T22</t>
+Đăng Khoa: review T24; chốt cách trình bày FD có điều kiện ở T22
+Đăng Khoa: review T27; T30 chốt TAI_KHOAN.vai_tro (giữ hay suy từ loai_nv)</t>
   </si>
   <si>
     <t>docs/5_anh-xa/T20_AnhXa_MangB.md
 commit 78857c7, nhánh Khoi
-docs/6_chuan-hoa/T24_FD_MangB.md</t>
+docs/6_chuan-hoa/T24_FD_MangB.md
+docs/6_chuan-hoa/T27_ChuanHoa_MangB.md</t>
   </si>
 </sst>
 </file>
@@ -3417,7 +3423,7 @@
       </c>
       <c r="L30" s="22"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12" ht="98" x14ac:dyDescent="0.2">
       <c r="A31" s="13" t="s">
         <v>118</v>
       </c>
@@ -3448,12 +3454,14 @@
         <v>120</v>
       </c>
       <c r="J31" s="20" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="K31" s="21">
-        <v>0</v>
-      </c>
-      <c r="L31" s="22"/>
+        <v>1</v>
+      </c>
+      <c r="L31" s="22" t="s">
+        <v>401</v>
+      </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="13" t="s">
@@ -4943,7 +4951,7 @@
         <v>8</v>
       </c>
       <c r="G12" s="20" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -5255,7 +5263,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="112" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="154" x14ac:dyDescent="0.2">
       <c r="A9" s="20">
         <v>4</v>
       </c>
@@ -5266,16 +5274,16 @@
         <v>22</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -6113,7 +6121,7 @@
       </c>
       <c r="C5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Hoàn thành")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Đang làm")</f>
@@ -6125,11 +6133,11 @@
       </c>
       <c r="F5" s="34">
         <f>IFERROR(C5/B5,0)</f>
-        <v>0.36842105263157893</v>
+        <v>0.42105263157894735</v>
       </c>
       <c r="G5" s="34">
         <f>IFERROR(AVERAGEIF('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.45789473684210524</v>
+        <v>0.51052631578947361</v>
       </c>
       <c r="H5" s="7">
         <f>COUNTIF('Kế hoạch'!$H$5:$H$109,A5)</f>
@@ -6245,7 +6253,7 @@
       </c>
       <c r="C9" s="35">
         <f>SUM(C5:C8)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D9" s="35">
         <f>SUM(D5:D8)</f>
@@ -6257,11 +6265,11 @@
       </c>
       <c r="F9" s="36">
         <f>IFERROR(C9/B9,0)</f>
-        <v>0.29090909090909089</v>
+        <v>0.30909090909090908</v>
       </c>
       <c r="G9" s="36">
         <f>IFERROR(AVERAGE('Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.32181818181818189</v>
+        <v>0.34</v>
       </c>
       <c r="H9" s="35">
         <f>SUM(H5:H8)</f>
@@ -6331,11 +6339,11 @@
       </c>
       <c r="C16" s="13">
         <f>COUNTIFS('Kế hoạch'!$E$5:$E$109,A16,'Kế hoạch'!$J$5:$J$109,"Hoàn thành")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" s="39">
         <f>IFERROR(C16/B16,0)</f>
-        <v>0.14285714285714285</v>
+        <v>0.21428571428571427</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
T33: DDL mảng B (sql/B_schema.sql); cập nhật kế hoạch
4 bảng benh_nhan, giay_chuyen_khoa, lich_hen, tai_khoan; CHECK theo hình
thức (8C), hạn giấy 30 ngày, chủ tài khoản; FK kép (ma_giay, ma_bn) cho
BR-B03; EXCLUDE gist chống trùng lịch bác sĩ, bệnh nhân (BR-B02); 4 index.
Chạy thử trên PG16 với bảng A giả lập: 17 ca vi phạm đều bị chặn.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khoile/Documents/PTIT/HK5/CSDL/telemedicine/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F582DAB-94D2-584F-B51A-17E84C7944A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C988CD3B-DBD9-B849-B9F7-AE810C782224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1200" yWindow="660" windowWidth="29040" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="407">
   <si>
     <t>Kế hoạch công việc theo tuần</t>
   </si>
@@ -1325,23 +1325,29 @@
     <t>docs/6_chuan-hoa/T27_ChuanHoa_MangB.md – 4 bảng đạt BCNF, không tách; lập luận riêng cho FD có điều kiện (cột UNIQUE cho phép NULL); vai_tro trùng loai_nv chuyển T30 (27/10); chờ Đăng Khoa review</t>
   </si>
   <si>
-    <t>T20: ánh xạ mảng B sang lược đồ quan hệ (Elmasri bước 1–8): 4 bảng, PK/FK, UNIQUE; phân lớp LICH_HEN chọn 8C; truy vết ERD → lược đồ, quy tắc còn lại cho cài đặt
-T24: FD và khóa ứng viên 4 bảng mảng B, ghi FD đã xét và loại; nêu 2 điểm cho T27/T30 (FD có điều kiện trên cột UNIQUE cho phép NULL; TAI_KHOAN.vai_tro trùng NHAN_VIEN.loai_nv)
-T27: chứng minh 1NF → BCNF 4 bảng mảng B, không phải tách; ghi các thiết kế đã tránh vi phạm 3NF</t>
-  </si>
-  <si>
     <t>T21: review ánh xạ mảng C. T29: điền từ điển dữ liệu bảng mảng B</t>
+  </si>
+  <si>
+    <t>sql/B_schema.sql – 4 bảng; CHECK hình thức (8C), hạn giấy 30 ngày, chủ tài khoản; FK kép (ma_giay, ma_bn) cho BR-B03; EXCLUDE gist chống trùng lịch bác sĩ, bệnh nhân (BR-B02); 4 index. Đã chạy thử trên PG16 với bảng A giả lập (27/10). Giả định khóa A kiểu INTEGER, BAC_SI theo 8A – chờ T18, T32</t>
   </si>
   <si>
     <t>Hữu Khoa: chốt phương án ánh xạ BAC_SI (8A hay 8C) ở T19 – ảnh hưởng FK ma_bac_si_lap → BAC_SI_DA_KHOA; review T20
 Đăng Khoa: review T24; chốt cách trình bày FD có điều kiện ở T22
-Đăng Khoa: review T27; T30 chốt TAI_KHOAN.vai_tro (giữ hay suy từ loai_nv)</t>
+Đăng Khoa: review T27; T30 chốt TAI_KHOAN.vai_tro (giữ hay suy từ loai_nv)
+Hữu Khoa: T18 chốt kiểu khóa (INTEGER identity), giá trị loai_nv trùng vai_tro (QUAN_TRI_NHAN_SU, QUAN_TRI_TAI_KHOAN, QUAN_TRI_DANH_MUC, BAC_SI, LE_TAN); review T33</t>
   </si>
   <si>
     <t>docs/5_anh-xa/T20_AnhXa_MangB.md
 commit 78857c7, nhánh Khoi
 docs/6_chuan-hoa/T24_FD_MangB.md
-docs/6_chuan-hoa/T27_ChuanHoa_MangB.md</t>
+docs/6_chuan-hoa/T27_ChuanHoa_MangB.md
+sql/B_schema.sql</t>
+  </si>
+  <si>
+    <t>T20: ánh xạ mảng B sang lược đồ quan hệ (Elmasri bước 1–8): 4 bảng, PK/FK, UNIQUE; phân lớp LICH_HEN chọn 8C; truy vết ERD → lược đồ, quy tắc còn lại cho cài đặt
+T24: FD và khóa ứng viên 4 bảng mảng B, ghi FD đã xét và loại; nêu 2 điểm cho T27/T30 (FD có điều kiện trên cột UNIQUE cho phép NULL; TAI_KHOAN.vai_tro trùng NHAN_VIEN.loai_nv)
+T27: chứng minh 1NF → BCNF 4 bảng mảng B, không phải tách; ghi các thiết kế đã tránh vi phạm 3NF
+T33 (làm sớm): DDL mảng B, chạy thử 17 ca vi phạm trên PG16 đều bị chặn</t>
   </si>
 </sst>
 </file>
@@ -3653,7 +3659,7 @@
       </c>
       <c r="L36" s="22"/>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" ht="140" x14ac:dyDescent="0.2">
       <c r="A37" s="15" t="s">
         <v>137</v>
       </c>
@@ -3684,12 +3690,14 @@
         <v>139</v>
       </c>
       <c r="J37" s="20" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="K37" s="21">
-        <v>0</v>
-      </c>
-      <c r="L37" s="22"/>
+        <v>1</v>
+      </c>
+      <c r="L37" s="22" t="s">
+        <v>403</v>
+      </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" s="15" t="s">
@@ -5263,7 +5271,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="154" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="210" x14ac:dyDescent="0.2">
       <c r="A9" s="20">
         <v>4</v>
       </c>
@@ -5274,10 +5282,10 @@
         <v>22</v>
       </c>
       <c r="D9" s="22" t="s">
+        <v>406</v>
+      </c>
+      <c r="E9" s="22" t="s">
         <v>402</v>
-      </c>
-      <c r="E9" s="22" t="s">
-        <v>403</v>
       </c>
       <c r="F9" s="22" t="s">
         <v>404</v>
@@ -6121,7 +6129,7 @@
       </c>
       <c r="C5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Hoàn thành")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Đang làm")</f>
@@ -6133,11 +6141,11 @@
       </c>
       <c r="F5" s="34">
         <f>IFERROR(C5/B5,0)</f>
-        <v>0.42105263157894735</v>
+        <v>0.47368421052631576</v>
       </c>
       <c r="G5" s="34">
         <f>IFERROR(AVERAGEIF('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.51052631578947361</v>
+        <v>0.56315789473684208</v>
       </c>
       <c r="H5" s="7">
         <f>COUNTIF('Kế hoạch'!$H$5:$H$109,A5)</f>
@@ -6253,7 +6261,7 @@
       </c>
       <c r="C9" s="35">
         <f>SUM(C5:C8)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D9" s="35">
         <f>SUM(D5:D8)</f>
@@ -6265,11 +6273,11 @@
       </c>
       <c r="F9" s="36">
         <f>IFERROR(C9/B9,0)</f>
-        <v>0.30909090909090908</v>
+        <v>0.32727272727272727</v>
       </c>
       <c r="G9" s="36">
         <f>IFERROR(AVERAGE('Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.34</v>
+        <v>0.35818181818181821</v>
       </c>
       <c r="H9" s="35">
         <f>SUM(H5:H8)</f>
@@ -6356,11 +6364,11 @@
       </c>
       <c r="C17" s="15">
         <f>COUNTIFS('Kế hoạch'!$E$5:$E$109,A17,'Kế hoạch'!$J$5:$J$109,"Hoàn thành")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="40">
         <f>IFERROR(C17/B17,0)</f>
-        <v>0</v>
+        <v>6.6666666666666666E-2</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
T37: trigger và view mảng B (sql/B_trigger_view.sql); cập nhật kế hoạch
trg_lich_hen_hop_le (BR-B01 trong ca; BR-B03 giấy đúng chuyên khoa, còn hạn,
miễn tái khám), trg_trang_thai_lich_hen (BR-B05), trg_tai_khoan_vai_tro
(BR-B09), trg_tai_khoan_khong_xoa (BR-B10); view v_lich_hen_hom_nay.
Chạy thử trên PG16 với bảng A giả lập: 17 ca vi phạm đều bị chặn.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khoile/Documents/PTIT/HK5/CSDL/telemedicine/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C988CD3B-DBD9-B849-B9F7-AE810C782224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9CFF579-AB18-5649-B41A-DEC5A05561E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1200" yWindow="660" windowWidth="29040" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="408">
   <si>
     <t>Kế hoạch công việc theo tuần</t>
   </si>
@@ -1331,23 +1331,29 @@
     <t>sql/B_schema.sql – 4 bảng; CHECK hình thức (8C), hạn giấy 30 ngày, chủ tài khoản; FK kép (ma_giay, ma_bn) cho BR-B03; EXCLUDE gist chống trùng lịch bác sĩ, bệnh nhân (BR-B02); 4 index. Đã chạy thử trên PG16 với bảng A giả lập (27/10). Giả định khóa A kiểu INTEGER, BAC_SI theo 8A – chờ T18, T32</t>
   </si>
   <si>
+    <t>sql/B_trigger_view.sql – trg_lich_hen_hop_le (BR-B01 trong ca; BR-B03 giấy đúng chuyên khoa, còn hạn, miễn tái khám), trg_trang_thai_lich_hen (BR-B05), trg_tai_khoan_vai_tro (BR-B09), trg_tai_khoan_khong_xoa (BR-B10); view v_lich_hen_hom_nay. Chạy thử PG16 với bảng A giả lập: 17 ca vi phạm đều bị chặn (27/10). Giả định cột ca_lam_viec, bac_si_chuyen_khoa – chờ T32</t>
+  </si>
+  <si>
+    <t>T20: ánh xạ mảng B sang lược đồ quan hệ (Elmasri bước 1–8): 4 bảng, PK/FK, UNIQUE; phân lớp LICH_HEN chọn 8C; truy vết ERD → lược đồ, quy tắc còn lại cho cài đặt
+T24: FD và khóa ứng viên 4 bảng mảng B, ghi FD đã xét và loại; nêu 2 điểm cho T27/T30 (FD có điều kiện trên cột UNIQUE cho phép NULL; TAI_KHOAN.vai_tro trùng NHAN_VIEN.loai_nv)
+T27: chứng minh 1NF → BCNF 4 bảng mảng B, không phải tách; ghi các thiết kế đã tránh vi phạm 3NF
+T33 (làm sớm): DDL mảng B, chạy thử 17 ca vi phạm trên PG16 đều bị chặn
+T37 (làm sớm): 4 trigger + view v_lich_hen_hom_nay mảng B, chạy thử 17 ca vi phạm đều bị chặn</t>
+  </si>
+  <si>
     <t>Hữu Khoa: chốt phương án ánh xạ BAC_SI (8A hay 8C) ở T19 – ảnh hưởng FK ma_bac_si_lap → BAC_SI_DA_KHOA; review T20
 Đăng Khoa: review T24; chốt cách trình bày FD có điều kiện ở T22
 Đăng Khoa: review T27; T30 chốt TAI_KHOAN.vai_tro (giữ hay suy từ loai_nv)
-Hữu Khoa: T18 chốt kiểu khóa (INTEGER identity), giá trị loai_nv trùng vai_tro (QUAN_TRI_NHAN_SU, QUAN_TRI_TAI_KHOAN, QUAN_TRI_DANH_MUC, BAC_SI, LE_TAN); review T33</t>
+Hữu Khoa: T18 chốt kiểu khóa (INTEGER identity), giá trị loai_nv trùng vai_tro (QUAN_TRI_NHAN_SU, QUAN_TRI_TAI_KHOAN, QUAN_TRI_DANH_MUC, BAC_SI, LE_TAN); review T33
+Đăng Khoa: review T37; T39 seed phải thêm lịch hẹn ở DA_DAT rồi UPDATE, lịch nằm trong ca, lịch chuyên khoa có giấy hoặc tái khám</t>
   </si>
   <si>
     <t>docs/5_anh-xa/T20_AnhXa_MangB.md
 commit 78857c7, nhánh Khoi
 docs/6_chuan-hoa/T24_FD_MangB.md
 docs/6_chuan-hoa/T27_ChuanHoa_MangB.md
-sql/B_schema.sql</t>
-  </si>
-  <si>
-    <t>T20: ánh xạ mảng B sang lược đồ quan hệ (Elmasri bước 1–8): 4 bảng, PK/FK, UNIQUE; phân lớp LICH_HEN chọn 8C; truy vết ERD → lược đồ, quy tắc còn lại cho cài đặt
-T24: FD và khóa ứng viên 4 bảng mảng B, ghi FD đã xét và loại; nêu 2 điểm cho T27/T30 (FD có điều kiện trên cột UNIQUE cho phép NULL; TAI_KHOAN.vai_tro trùng NHAN_VIEN.loai_nv)
-T27: chứng minh 1NF → BCNF 4 bảng mảng B, không phải tách; ghi các thiết kế đã tránh vi phạm 3NF
-T33 (làm sớm): DDL mảng B, chạy thử 17 ca vi phạm trên PG16 đều bị chặn</t>
+sql/B_schema.sql
+sql/B_trigger_view.sql</t>
   </si>
 </sst>
 </file>
@@ -3844,12 +3850,14 @@
         <v>151</v>
       </c>
       <c r="J41" s="20" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="K41" s="21">
-        <v>0</v>
-      </c>
-      <c r="L41" s="22"/>
+        <v>1</v>
+      </c>
+      <c r="L41" s="22" t="s">
+        <v>404</v>
+      </c>
     </row>
     <row r="42" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="15" t="s">
@@ -5271,7 +5279,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="210" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="266" x14ac:dyDescent="0.2">
       <c r="A9" s="20">
         <v>4</v>
       </c>
@@ -5282,16 +5290,16 @@
         <v>22</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E9" s="22" t="s">
         <v>402</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -6129,7 +6137,7 @@
       </c>
       <c r="C5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Hoàn thành")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Đang làm")</f>
@@ -6141,11 +6149,11 @@
       </c>
       <c r="F5" s="34">
         <f>IFERROR(C5/B5,0)</f>
-        <v>0.47368421052631576</v>
+        <v>0.52631578947368418</v>
       </c>
       <c r="G5" s="34">
         <f>IFERROR(AVERAGEIF('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.56315789473684208</v>
+        <v>0.61578947368421044</v>
       </c>
       <c r="H5" s="7">
         <f>COUNTIF('Kế hoạch'!$H$5:$H$109,A5)</f>
@@ -6261,7 +6269,7 @@
       </c>
       <c r="C9" s="35">
         <f>SUM(C5:C8)</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D9" s="35">
         <f>SUM(D5:D8)</f>
@@ -6273,11 +6281,11 @@
       </c>
       <c r="F9" s="36">
         <f>IFERROR(C9/B9,0)</f>
-        <v>0.32727272727272727</v>
+        <v>0.34545454545454546</v>
       </c>
       <c r="G9" s="36">
         <f>IFERROR(AVERAGE('Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.35818181818181821</v>
+        <v>0.3763636363636364</v>
       </c>
       <c r="H9" s="35">
         <f>SUM(H5:H8)</f>
@@ -6364,11 +6372,11 @@
       </c>
       <c r="C17" s="15">
         <f>COUNTIFS('Kế hoạch'!$E$5:$E$109,A17,'Kế hoạch'!$J$5:$J$109,"Hoàn thành")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="40">
         <f>IFERROR(C17/B17,0)</f>
-        <v>6.6666666666666666E-2</v>
+        <v>0.13333333333333333</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
T30: rà phần B mục 2.2, 2.3, kiểm tra lại T33, T37; sửa T20, làm rõ T08; cập nhật kế hoạch
Đối chiếu T20, T24, T27 với B_schema.sql, B_trigger_view.sql. L01: T20 ghi
khóa ngoại kép (ma_giay, ma_bn) như DDL. L02–L05: T08 mục 5 ghi rõ giấy
còn hạn theo ngày hẹn, giấy chỉ cho lịch chuyên khoa, lịch ở trạng thái cuối
không sửa được, giấy gắn với lịch đã hủy/vắng mặt coi là đã dùng. Bảng quy
tắc → cơ chế; C1–C4 chờ nhóm chốt. Phần A, C chờ.

Kiểm tra lại T33, T37: chặn TRUNCATE tai_khoan (BR-B10); CREATE OR REPLACE
TRIGGER để chạy lại được; báo lỗi BR-B03 khi dùng lại giấy; sửa comment
đầu B_schema.sql, ghi chú khóa tự tăng cho dữ liệu mẫu.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khoile/Documents/PTIT/HK5/CSDL/telemedicine/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9CFF579-AB18-5649-B41A-DEC5A05561E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E23F4AB-384C-0B42-8064-9E682855A93A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1200" yWindow="660" windowWidth="29040" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="409">
   <si>
     <t>Kế hoạch công việc theo tuần</t>
   </si>
@@ -1338,14 +1338,8 @@
 T24: FD và khóa ứng viên 4 bảng mảng B, ghi FD đã xét và loại; nêu 2 điểm cho T27/T30 (FD có điều kiện trên cột UNIQUE cho phép NULL; TAI_KHOAN.vai_tro trùng NHAN_VIEN.loai_nv)
 T27: chứng minh 1NF → BCNF 4 bảng mảng B, không phải tách; ghi các thiết kế đã tránh vi phạm 3NF
 T33 (làm sớm): DDL mảng B, chạy thử 17 ca vi phạm trên PG16 đều bị chặn
-T37 (làm sớm): 4 trigger + view v_lich_hen_hom_nay mảng B, chạy thử 17 ca vi phạm đều bị chặn</t>
-  </si>
-  <si>
-    <t>Hữu Khoa: chốt phương án ánh xạ BAC_SI (8A hay 8C) ở T19 – ảnh hưởng FK ma_bac_si_lap → BAC_SI_DA_KHOA; review T20
-Đăng Khoa: review T24; chốt cách trình bày FD có điều kiện ở T22
-Đăng Khoa: review T27; T30 chốt TAI_KHOAN.vai_tro (giữ hay suy từ loai_nv)
-Hữu Khoa: T18 chốt kiểu khóa (INTEGER identity), giá trị loai_nv trùng vai_tro (QUAN_TRI_NHAN_SU, QUAN_TRI_TAI_KHOAN, QUAN_TRI_DANH_MUC, BAC_SI, LE_TAN); review T33
-Đăng Khoa: review T37; T39 seed phải thêm lịch hẹn ở DA_DAT rồi UPDATE, lịch nằm trong ca, lịch chuyên khoa có giấy hoặc tái khám</t>
+T37 (làm sớm): 4 trigger + view v_lich_hen_hom_nay mảng B, chạy thử 17 ca vi phạm đều bị chặn
+T30 (phần B): đối chiếu T20, T24, T27 với DDL, trigger; sửa T20 (FK kép giấy – bệnh nhân); lập danh sách lỗi, bảng quy tắc → cơ chế</t>
   </si>
   <si>
     <t>docs/5_anh-xa/T20_AnhXa_MangB.md
@@ -1353,7 +1347,19 @@
 docs/6_chuan-hoa/T24_FD_MangB.md
 docs/6_chuan-hoa/T27_ChuanHoa_MangB.md
 sql/B_schema.sql
-sql/B_trigger_view.sql</t>
+sql/B_trigger_view.sql
+docs/6_chuan-hoa/T30_ReviewCheo.md</t>
+  </si>
+  <si>
+    <t>docs/6_chuan-hoa/T30_ReviewCheo.md – đã rà phần B (Khôi, 27/10): L01 sửa T20 (FK kép giấy – bệnh nhân); L02–L04 diễn giải trigger đã xác nhận, ghi vào T08 mục 5; ERD B không phải sửa; chờ A, C (T19, T21, T26, T28), mục 3 (T29); C1 vai_tro/loai_nv chờ nhóm họp</t>
+  </si>
+  <si>
+    <t>Hữu Khoa: chốt phương án ánh xạ BAC_SI (8A hay 8C) ở T19 – ảnh hưởng FK ma_bac_si_lap → BAC_SI_DA_KHOA; review T20
+Đăng Khoa: review T24; chốt cách trình bày FD có điều kiện ở T22
+Đăng Khoa: review T27; T30 chốt TAI_KHOAN.vai_tro (giữ hay suy từ loai_nv)
+Hữu Khoa: T18 chốt kiểu khóa (INTEGER identity), giá trị loai_nv trùng vai_tro (QUAN_TRI_NHAN_SU, QUAN_TRI_TAI_KHOAN, QUAN_TRI_DANH_MUC, BAC_SI, LE_TAN); review T33
+Đăng Khoa: review T37; T39 seed phải thêm lịch hẹn ở DA_DAT rồi UPDATE, lịch nằm trong ca, lịch chuyên khoa có giấy hoặc tái khám
+Cả nhóm: họp chốt C1 (TAI_KHOAN.vai_tro trùng loai_nv, BR-B10 đổi vai trò mâu thuẫn BR-A09)</t>
   </si>
 </sst>
 </file>
@@ -3582,12 +3588,14 @@
         <v>129</v>
       </c>
       <c r="J34" s="20" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="K34" s="21">
-        <v>0</v>
-      </c>
-      <c r="L34" s="22"/>
+        <v>0.3</v>
+      </c>
+      <c r="L34" s="22" t="s">
+        <v>407</v>
+      </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="13" t="s">
@@ -5279,7 +5287,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="266" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="306" x14ac:dyDescent="0.2">
       <c r="A9" s="20">
         <v>4</v>
       </c>
@@ -5296,10 +5304,10 @@
         <v>402</v>
       </c>
       <c r="F9" s="22" t="s">
+        <v>408</v>
+      </c>
+      <c r="G9" s="22" t="s">
         <v>406</v>
-      </c>
-      <c r="G9" s="22" t="s">
-        <v>407</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -6207,7 +6215,7 @@
       </c>
       <c r="D7" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A7,'Kế hoạch'!$J$5:$J$109,"Đang làm")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A7,'Kế hoạch'!$J$5:$J$109,"Trễ hạn")</f>
@@ -6219,7 +6227,7 @@
       </c>
       <c r="G7" s="34">
         <f>IFERROR(AVERAGEIF('Kế hoạch'!$G$5:$G$109,A7,'Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.23529411764705882</v>
+        <v>0.25294117647058822</v>
       </c>
       <c r="H7" s="7">
         <f>COUNTIF('Kế hoạch'!$H$5:$H$109,A7)</f>
@@ -6273,7 +6281,7 @@
       </c>
       <c r="D9" s="35">
         <f>SUM(D5:D8)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" s="35">
         <f>SUM(E5:E8)</f>
@@ -6285,7 +6293,7 @@
       </c>
       <c r="G9" s="36">
         <f>IFERROR(AVERAGE('Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.3763636363636364</v>
+        <v>0.38181818181818189</v>
       </c>
       <c r="H9" s="35">
         <f>SUM(H5:H8)</f>

</xml_diff>

<commit_message>
T41: 4 truy vấn phức tạp mảng B (sql/queries_B.sql); cập nhật kế hoạch
Q1 tỷ lệ hủy/vắng mặt theo bác sĩ (JOIN, FILTER, HAVING); Q2 doanh thu
theo chuyên khoa theo tháng (hàm cửa sổ); Q3 bệnh nhân khám > 3 lần trong
6 tháng (subquery FROM, EXISTS tương quan); Q4 khung giờ đông nhất, tỷ lệ
từ xa (ROLLUP, RANK). Kiểm chứng trên dữ liệu thử đi qua trigger, đối
chiếu với tính độc lập: khớp.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khoile/Documents/PTIT/HK5/CSDL/telemedicine/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E23F4AB-384C-0B42-8064-9E682855A93A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C6B8CB6-03CC-AA4F-BD28-6C2E99BCAAB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1200" yWindow="660" windowWidth="29040" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="410">
   <si>
     <t>Kế hoạch công việc theo tuần</t>
   </si>
@@ -1334,12 +1334,27 @@
     <t>sql/B_trigger_view.sql – trg_lich_hen_hop_le (BR-B01 trong ca; BR-B03 giấy đúng chuyên khoa, còn hạn, miễn tái khám), trg_trang_thai_lich_hen (BR-B05), trg_tai_khoan_vai_tro (BR-B09), trg_tai_khoan_khong_xoa (BR-B10); view v_lich_hen_hom_nay. Chạy thử PG16 với bảng A giả lập: 17 ca vi phạm đều bị chặn (27/10). Giả định cột ca_lam_viec, bac_si_chuyen_khoa – chờ T32</t>
   </si>
   <si>
+    <t>docs/6_chuan-hoa/T30_ReviewCheo.md – đã rà phần B (Khôi, 27/10): L01 sửa T20 (FK kép giấy – bệnh nhân); L02–L04 diễn giải trigger đã xác nhận, ghi vào T08 mục 5; ERD B không phải sửa; chờ A, C (T19, T21, T26, T28), mục 3 (T29); C1 vai_tro/loai_nv chờ nhóm họp</t>
+  </si>
+  <si>
+    <t>Hữu Khoa: chốt phương án ánh xạ BAC_SI (8A hay 8C) ở T19 – ảnh hưởng FK ma_bac_si_lap → BAC_SI_DA_KHOA; review T20
+Đăng Khoa: review T24; chốt cách trình bày FD có điều kiện ở T22
+Đăng Khoa: review T27; T30 chốt TAI_KHOAN.vai_tro (giữ hay suy từ loai_nv)
+Hữu Khoa: T18 chốt kiểu khóa (INTEGER identity), giá trị loai_nv trùng vai_tro (QUAN_TRI_NHAN_SU, QUAN_TRI_TAI_KHOAN, QUAN_TRI_DANH_MUC, BAC_SI, LE_TAN); review T33
+Đăng Khoa: review T37; T39 seed phải thêm lịch hẹn ở DA_DAT rồi UPDATE, lịch nằm trong ca, lịch chuyên khoa có giấy hoặc tái khám
+Cả nhóm: họp chốt C1 (TAI_KHOAN.vai_tro trùng loai_nv, BR-B10 đổi vai trò mâu thuẫn BR-A09)</t>
+  </si>
+  <si>
+    <t>sql/queries_B.sql – Q1 tỷ lệ hủy/vắng theo bác sĩ (JOIN, FILTER, HAVING); Q2 doanh thu chuyên khoa theo tháng (hàm cửa sổ); Q3 bệnh nhân &gt; 3 lần khám/6 tháng (subquery FROM + EXISTS tương quan); Q4 khung giờ đông nhất, tỷ lệ từ xa (ROLLUP, RANK). Kiểm chứng trên dữ liệu thử qua trigger, đối chiếu tính độc lập bằng Python: khớp (27/10). Chờ Đăng Khoa review</t>
+  </si>
+  <si>
     <t>T20: ánh xạ mảng B sang lược đồ quan hệ (Elmasri bước 1–8): 4 bảng, PK/FK, UNIQUE; phân lớp LICH_HEN chọn 8C; truy vết ERD → lược đồ, quy tắc còn lại cho cài đặt
 T24: FD và khóa ứng viên 4 bảng mảng B, ghi FD đã xét và loại; nêu 2 điểm cho T27/T30 (FD có điều kiện trên cột UNIQUE cho phép NULL; TAI_KHOAN.vai_tro trùng NHAN_VIEN.loai_nv)
 T27: chứng minh 1NF → BCNF 4 bảng mảng B, không phải tách; ghi các thiết kế đã tránh vi phạm 3NF
 T33 (làm sớm): DDL mảng B, chạy thử 17 ca vi phạm trên PG16 đều bị chặn
 T37 (làm sớm): 4 trigger + view v_lich_hen_hom_nay mảng B, chạy thử 17 ca vi phạm đều bị chặn
-T30 (phần B): đối chiếu T20, T24, T27 với DDL, trigger; sửa T20 (FK kép giấy – bệnh nhân); lập danh sách lỗi, bảng quy tắc → cơ chế</t>
+T30 (phần B): đối chiếu T20, T24, T27 với DDL, trigger; sửa T20 (FK kép giấy – bệnh nhân); lập danh sách lỗi, bảng quy tắc → cơ chế
+T41 (làm sớm): 4 truy vấn mảng B, kiểm chứng trên dữ liệu thử đi qua trigger</t>
   </si>
   <si>
     <t>docs/5_anh-xa/T20_AnhXa_MangB.md
@@ -1348,18 +1363,8 @@
 docs/6_chuan-hoa/T27_ChuanHoa_MangB.md
 sql/B_schema.sql
 sql/B_trigger_view.sql
-docs/6_chuan-hoa/T30_ReviewCheo.md</t>
-  </si>
-  <si>
-    <t>docs/6_chuan-hoa/T30_ReviewCheo.md – đã rà phần B (Khôi, 27/10): L01 sửa T20 (FK kép giấy – bệnh nhân); L02–L04 diễn giải trigger đã xác nhận, ghi vào T08 mục 5; ERD B không phải sửa; chờ A, C (T19, T21, T26, T28), mục 3 (T29); C1 vai_tro/loai_nv chờ nhóm họp</t>
-  </si>
-  <si>
-    <t>Hữu Khoa: chốt phương án ánh xạ BAC_SI (8A hay 8C) ở T19 – ảnh hưởng FK ma_bac_si_lap → BAC_SI_DA_KHOA; review T20
-Đăng Khoa: review T24; chốt cách trình bày FD có điều kiện ở T22
-Đăng Khoa: review T27; T30 chốt TAI_KHOAN.vai_tro (giữ hay suy từ loai_nv)
-Hữu Khoa: T18 chốt kiểu khóa (INTEGER identity), giá trị loai_nv trùng vai_tro (QUAN_TRI_NHAN_SU, QUAN_TRI_TAI_KHOAN, QUAN_TRI_DANH_MUC, BAC_SI, LE_TAN); review T33
-Đăng Khoa: review T37; T39 seed phải thêm lịch hẹn ở DA_DAT rồi UPDATE, lịch nằm trong ca, lịch chuyên khoa có giấy hoặc tái khám
-Cả nhóm: họp chốt C1 (TAI_KHOAN.vai_tro trùng loai_nv, BR-B10 đổi vai trò mâu thuẫn BR-A09)</t>
+docs/6_chuan-hoa/T30_ReviewCheo.md
+sql/queries_B.sql</t>
   </si>
 </sst>
 </file>
@@ -3594,7 +3599,7 @@
         <v>0.3</v>
       </c>
       <c r="L34" s="22" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
@@ -3981,7 +3986,7 @@
       </c>
       <c r="L44" s="22"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:12" ht="182" x14ac:dyDescent="0.2">
       <c r="A45" s="15" t="s">
         <v>161</v>
       </c>
@@ -4012,12 +4017,14 @@
         <v>163</v>
       </c>
       <c r="J45" s="20" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="K45" s="21">
-        <v>0</v>
-      </c>
-      <c r="L45" s="22"/>
+        <v>1</v>
+      </c>
+      <c r="L45" s="22" t="s">
+        <v>407</v>
+      </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" s="15" t="s">
@@ -5298,16 +5305,16 @@
         <v>22</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="E9" s="22" t="s">
         <v>402</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -6145,7 +6152,7 @@
       </c>
       <c r="C5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Hoàn thành")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Đang làm")</f>
@@ -6157,11 +6164,11 @@
       </c>
       <c r="F5" s="34">
         <f>IFERROR(C5/B5,0)</f>
-        <v>0.52631578947368418</v>
+        <v>0.57894736842105265</v>
       </c>
       <c r="G5" s="34">
         <f>IFERROR(AVERAGEIF('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.61578947368421044</v>
+        <v>0.66842105263157892</v>
       </c>
       <c r="H5" s="7">
         <f>COUNTIF('Kế hoạch'!$H$5:$H$109,A5)</f>
@@ -6277,7 +6284,7 @@
       </c>
       <c r="C9" s="35">
         <f>SUM(C5:C8)</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D9" s="35">
         <f>SUM(D5:D8)</f>
@@ -6289,11 +6296,11 @@
       </c>
       <c r="F9" s="36">
         <f>IFERROR(C9/B9,0)</f>
-        <v>0.34545454545454546</v>
+        <v>0.36363636363636365</v>
       </c>
       <c r="G9" s="36">
         <f>IFERROR(AVERAGE('Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.38181818181818189</v>
+        <v>0.40000000000000008</v>
       </c>
       <c r="H9" s="35">
         <f>SUM(H5:H8)</f>
@@ -6380,11 +6387,11 @@
       </c>
       <c r="C17" s="15">
         <f>COUNTIFS('Kế hoạch'!$E$5:$E$109,A17,'Kế hoạch'!$J$5:$J$109,"Hoàn thành")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D17" s="40">
         <f>IFERROR(C17/B17,0)</f>
-        <v>0.13333333333333333</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
T17: hoàn thành, nộp báo cáo v2.1 ngày 21/10/2026
Điền ngày nộp trên trang bìa báo cáo v2.1; kế hoạch: T17 hoàn thành, 100%.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khoile/Documents/PTIT/HK5/CSDL/telemedicine/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C6B8CB6-03CC-AA4F-BD28-6C2E99BCAAB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABCFF4B7-E797-124B-BDC6-E0973C12BA8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1200" yWindow="660" windowWidth="29040" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -334,9 +334,6 @@
     <t>Báo cáo v2.1</t>
   </si>
   <si>
-    <t>docs/INT1313_TX_G5_DeTai05_Telemedicine_v2.1.docx – mục Giới thiệu tóm tắt, 1, 1.2, 2, 2.1 hoàn chỉnh, có ERD tổng; còn review chéo, điền ngày nộp, nộp</t>
-  </si>
-  <si>
     <t>T18</t>
   </si>
   <si>
@@ -1365,6 +1362,9 @@
 sql/B_trigger_view.sql
 docs/6_chuan-hoa/T30_ReviewCheo.md
 sql/queries_B.sql</t>
+  </si>
+  <si>
+    <t>docs/INT1313_TX_G5_DeTai05_Telemedicine_v2.1.docx – mục Giới thiệu tóm tắt, 1, 1.2, 2, 2.1 hoàn chỉnh, có ERD tổng; đã nộp 21/10/2026</t>
   </si>
 </sst>
 </file>
@@ -1992,46 +1992,46 @@
   <sheetData>
     <row r="1" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>216</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -2039,19 +2039,19 @@
         <v>22</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="E8" s="8" t="s">
         <v>220</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="F8" s="8" t="s">
         <v>221</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -2059,19 +2059,19 @@
         <v>34</v>
       </c>
       <c r="B9" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>223</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="D9" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="E9" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="F9" s="8" t="s">
         <v>226</v>
-      </c>
-      <c r="F9" s="8" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.2">
@@ -2079,24 +2079,24 @@
         <v>28</v>
       </c>
       <c r="B10" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="D10" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="E10" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="F10" s="8" t="s">
         <v>231</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="42" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B11" s="43"/>
       <c r="C11" s="43"/>
@@ -2106,7 +2106,7 @@
     </row>
     <row r="13" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -2120,13 +2120,13 @@
         <v>3</v>
       </c>
       <c r="D14" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="E14" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="6" t="s">
         <v>236</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
@@ -2134,19 +2134,19 @@
         <v>15</v>
       </c>
       <c r="B15" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>238</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="D15" s="10" t="s">
         <v>239</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="E15" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="F15" s="9" t="s">
         <v>241</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
@@ -2154,92 +2154,92 @@
         <v>62</v>
       </c>
       <c r="B16" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="C16" s="11" t="s">
         <v>243</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="D16" s="12" t="s">
         <v>244</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="E16" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="F16" s="11" t="s">
         <v>246</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B17" s="14" t="s">
+        <v>247</v>
+      </c>
+      <c r="C17" s="13" t="s">
         <v>248</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="D17" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="E17" s="14" t="s">
         <v>250</v>
       </c>
-      <c r="E17" s="14" t="s">
+      <c r="F17" s="13" t="s">
         <v>251</v>
-      </c>
-      <c r="F17" s="13" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B18" s="16" t="s">
+        <v>252</v>
+      </c>
+      <c r="C18" s="15" t="s">
         <v>253</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="D18" s="16" t="s">
         <v>254</v>
       </c>
-      <c r="D18" s="16" t="s">
+      <c r="E18" s="16" t="s">
         <v>255</v>
       </c>
-      <c r="E18" s="16" t="s">
+      <c r="F18" s="15" t="s">
         <v>256</v>
-      </c>
-      <c r="F18" s="15" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B19" s="18" t="s">
+        <v>257</v>
+      </c>
+      <c r="C19" s="17" t="s">
         <v>258</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="D19" s="18" t="s">
         <v>259</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="E19" s="18" t="s">
         <v>260</v>
       </c>
-      <c r="E19" s="18" t="s">
+      <c r="F19" s="17" t="s">
         <v>261</v>
-      </c>
-      <c r="F19" s="17" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B22" s="44" t="s">
         <v>264</v>
-      </c>
-      <c r="B22" s="44" t="s">
-        <v>265</v>
       </c>
       <c r="C22" s="43"/>
       <c r="D22" s="43"/>
@@ -2248,10 +2248,10 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="B23" s="44" t="s">
         <v>266</v>
-      </c>
-      <c r="B23" s="44" t="s">
-        <v>267</v>
       </c>
       <c r="C23" s="43"/>
       <c r="D23" s="43"/>
@@ -2260,10 +2260,10 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="B24" s="44" t="s">
         <v>268</v>
-      </c>
-      <c r="B24" s="44" t="s">
-        <v>269</v>
       </c>
       <c r="C24" s="43"/>
       <c r="D24" s="43"/>
@@ -2272,10 +2272,10 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="B25" s="44" t="s">
         <v>270</v>
-      </c>
-      <c r="B25" s="44" t="s">
-        <v>271</v>
       </c>
       <c r="C25" s="43"/>
       <c r="D25" s="43"/>
@@ -2284,10 +2284,10 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="B26" s="44" t="s">
         <v>272</v>
-      </c>
-      <c r="B26" s="44" t="s">
-        <v>273</v>
       </c>
       <c r="C26" s="43"/>
       <c r="D26" s="43"/>
@@ -2296,12 +2296,12 @@
     </row>
     <row r="28" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="44" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B29" s="43"/>
       <c r="C29" s="43"/>
@@ -2311,7 +2311,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="44" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B30" s="43"/>
       <c r="C30" s="43"/>
@@ -2321,7 +2321,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="44" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B31" s="43"/>
       <c r="C31" s="43"/>
@@ -2331,7 +2331,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="44" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B32" s="43"/>
       <c r="C32" s="43"/>
@@ -3091,18 +3091,18 @@
         <v>88</v>
       </c>
       <c r="J21" s="20" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="K21" s="21">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="L21" s="22" t="s">
-        <v>89</v>
+        <v>409</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B22" s="13">
         <v>5</v>
@@ -3116,10 +3116,10 @@
         <v/>
       </c>
       <c r="E22" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="F22" s="14" t="s">
         <v>91</v>
-      </c>
-      <c r="F22" s="14" t="s">
-        <v>92</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>34</v>
@@ -3128,7 +3128,7 @@
         <v>17</v>
       </c>
       <c r="I22" s="14" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J22" s="20" t="s">
         <v>19</v>
@@ -3140,7 +3140,7 @@
     </row>
     <row r="23" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B23" s="13">
         <v>5</v>
@@ -3154,10 +3154,10 @@
         <v/>
       </c>
       <c r="E23" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F23" s="14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G23" s="13" t="s">
         <v>34</v>
@@ -3166,7 +3166,7 @@
         <v>28</v>
       </c>
       <c r="I23" s="14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J23" s="20" t="s">
         <v>19</v>
@@ -3178,7 +3178,7 @@
     </row>
     <row r="24" spans="1:12" ht="126" x14ac:dyDescent="0.2">
       <c r="A24" s="13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B24" s="13">
         <v>5</v>
@@ -3192,10 +3192,10 @@
         <v/>
       </c>
       <c r="E24" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G24" s="13" t="s">
         <v>22</v>
@@ -3204,7 +3204,7 @@
         <v>34</v>
       </c>
       <c r="I24" s="14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J24" s="20" t="s">
         <v>30</v>
@@ -3213,12 +3213,12 @@
         <v>1</v>
       </c>
       <c r="L24" s="22" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B25" s="13">
         <v>5</v>
@@ -3232,10 +3232,10 @@
         <v/>
       </c>
       <c r="E25" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F25" s="14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G25" s="13" t="s">
         <v>28</v>
@@ -3244,7 +3244,7 @@
         <v>22</v>
       </c>
       <c r="I25" s="14" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J25" s="20" t="s">
         <v>19</v>
@@ -3256,7 +3256,7 @@
     </row>
     <row r="26" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B26" s="13">
         <v>6</v>
@@ -3270,10 +3270,10 @@
         <v/>
       </c>
       <c r="E26" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G26" s="13" t="s">
         <v>28</v>
@@ -3282,7 +3282,7 @@
         <v>22</v>
       </c>
       <c r="I26" s="14" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J26" s="20" t="s">
         <v>19</v>
@@ -3294,7 +3294,7 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B27" s="13">
         <v>6</v>
@@ -3308,10 +3308,10 @@
         <v/>
       </c>
       <c r="E27" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G27" s="13" t="s">
         <v>34</v>
@@ -3320,7 +3320,7 @@
         <v>28</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="J27" s="20" t="s">
         <v>19</v>
@@ -3332,7 +3332,7 @@
     </row>
     <row r="28" spans="1:12" ht="98" x14ac:dyDescent="0.2">
       <c r="A28" s="13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B28" s="13">
         <v>6</v>
@@ -3346,10 +3346,10 @@
         <v/>
       </c>
       <c r="E28" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G28" s="13" t="s">
         <v>22</v>
@@ -3358,7 +3358,7 @@
         <v>28</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J28" s="20" t="s">
         <v>30</v>
@@ -3367,12 +3367,12 @@
         <v>1</v>
       </c>
       <c r="L28" s="22" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B29" s="13">
         <v>6</v>
@@ -3386,10 +3386,10 @@
         <v/>
       </c>
       <c r="E29" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G29" s="13" t="s">
         <v>28</v>
@@ -3398,7 +3398,7 @@
         <v>34</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J29" s="20" t="s">
         <v>19</v>
@@ -3410,7 +3410,7 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B30" s="13">
         <v>7</v>
@@ -3424,10 +3424,10 @@
         <v/>
       </c>
       <c r="E30" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F30" s="14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G30" s="13" t="s">
         <v>34</v>
@@ -3436,7 +3436,7 @@
         <v>28</v>
       </c>
       <c r="I30" s="14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J30" s="20" t="s">
         <v>19</v>
@@ -3448,7 +3448,7 @@
     </row>
     <row r="31" spans="1:12" ht="98" x14ac:dyDescent="0.2">
       <c r="A31" s="13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B31" s="13">
         <v>7</v>
@@ -3462,10 +3462,10 @@
         <v/>
       </c>
       <c r="E31" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G31" s="13" t="s">
         <v>22</v>
@@ -3474,7 +3474,7 @@
         <v>28</v>
       </c>
       <c r="I31" s="14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J31" s="20" t="s">
         <v>30</v>
@@ -3483,12 +3483,12 @@
         <v>1</v>
       </c>
       <c r="L31" s="22" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B32" s="13">
         <v>7</v>
@@ -3502,10 +3502,10 @@
         <v/>
       </c>
       <c r="E32" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F32" s="14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G32" s="13" t="s">
         <v>28</v>
@@ -3514,7 +3514,7 @@
         <v>34</v>
       </c>
       <c r="I32" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J32" s="20" t="s">
         <v>19</v>
@@ -3526,7 +3526,7 @@
     </row>
     <row r="33" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="13" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B33" s="13">
         <v>7</v>
@@ -3540,10 +3540,10 @@
         <v/>
       </c>
       <c r="E33" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G33" s="13" t="s">
         <v>34</v>
@@ -3552,7 +3552,7 @@
         <v>17</v>
       </c>
       <c r="I33" s="14" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J33" s="20" t="s">
         <v>19</v>
@@ -3564,7 +3564,7 @@
     </row>
     <row r="34" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B34" s="13">
         <v>8</v>
@@ -3578,10 +3578,10 @@
         <v/>
       </c>
       <c r="E34" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G34" s="13" t="s">
         <v>28</v>
@@ -3590,7 +3590,7 @@
         <v>17</v>
       </c>
       <c r="I34" s="14" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J34" s="20" t="s">
         <v>24</v>
@@ -3599,12 +3599,12 @@
         <v>0.3</v>
       </c>
       <c r="L34" s="22" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B35" s="13">
         <v>8</v>
@@ -3618,10 +3618,10 @@
         <v/>
       </c>
       <c r="E35" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G35" s="13" t="s">
         <v>22</v>
@@ -3630,7 +3630,7 @@
         <v>17</v>
       </c>
       <c r="I35" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J35" s="20" t="s">
         <v>19</v>
@@ -3642,7 +3642,7 @@
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B36" s="15">
         <v>9</v>
@@ -3656,10 +3656,10 @@
         <v/>
       </c>
       <c r="E36" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F36" s="16" t="s">
         <v>134</v>
-      </c>
-      <c r="F36" s="16" t="s">
-        <v>135</v>
       </c>
       <c r="G36" s="15" t="s">
         <v>34</v>
@@ -3668,7 +3668,7 @@
         <v>28</v>
       </c>
       <c r="I36" s="16" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J36" s="20" t="s">
         <v>19</v>
@@ -3680,7 +3680,7 @@
     </row>
     <row r="37" spans="1:12" ht="140" x14ac:dyDescent="0.2">
       <c r="A37" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B37" s="15">
         <v>9</v>
@@ -3694,10 +3694,10 @@
         <v/>
       </c>
       <c r="E37" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F37" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G37" s="15" t="s">
         <v>22</v>
@@ -3706,7 +3706,7 @@
         <v>34</v>
       </c>
       <c r="I37" s="16" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J37" s="20" t="s">
         <v>30</v>
@@ -3715,12 +3715,12 @@
         <v>1</v>
       </c>
       <c r="L37" s="22" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A38" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B38" s="15">
         <v>9</v>
@@ -3734,10 +3734,10 @@
         <v/>
       </c>
       <c r="E38" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F38" s="16" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G38" s="15" t="s">
         <v>28</v>
@@ -3746,7 +3746,7 @@
         <v>22</v>
       </c>
       <c r="I38" s="16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J38" s="20" t="s">
         <v>19</v>
@@ -3758,7 +3758,7 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A39" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B39" s="15">
         <v>9</v>
@@ -3772,10 +3772,10 @@
         <v/>
       </c>
       <c r="E39" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F39" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G39" s="15" t="s">
         <v>34</v>
@@ -3784,7 +3784,7 @@
         <v>17</v>
       </c>
       <c r="I39" s="16" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J39" s="20" t="s">
         <v>19</v>
@@ -3796,7 +3796,7 @@
     </row>
     <row r="40" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B40" s="15">
         <v>9</v>
@@ -3810,10 +3810,10 @@
         <v/>
       </c>
       <c r="E40" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G40" s="15" t="s">
         <v>34</v>
@@ -3822,7 +3822,7 @@
         <v>28</v>
       </c>
       <c r="I40" s="16" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J40" s="20" t="s">
         <v>19</v>
@@ -3834,7 +3834,7 @@
     </row>
     <row r="41" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="15" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B41" s="15">
         <v>9</v>
@@ -3848,10 +3848,10 @@
         <v/>
       </c>
       <c r="E41" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F41" s="16" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G41" s="15" t="s">
         <v>22</v>
@@ -3860,7 +3860,7 @@
         <v>28</v>
       </c>
       <c r="I41" s="16" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J41" s="20" t="s">
         <v>30</v>
@@ -3869,12 +3869,12 @@
         <v>1</v>
       </c>
       <c r="L41" s="22" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B42" s="15">
         <v>9</v>
@@ -3888,10 +3888,10 @@
         <v/>
       </c>
       <c r="E42" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F42" s="16" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G42" s="15" t="s">
         <v>28</v>
@@ -3900,7 +3900,7 @@
         <v>34</v>
       </c>
       <c r="I42" s="16" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J42" s="20" t="s">
         <v>19</v>
@@ -3912,7 +3912,7 @@
     </row>
     <row r="43" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B43" s="15">
         <v>9</v>
@@ -3926,10 +3926,10 @@
         <v/>
       </c>
       <c r="E43" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F43" s="16" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G43" s="15" t="s">
         <v>28</v>
@@ -3938,7 +3938,7 @@
         <v>17</v>
       </c>
       <c r="I43" s="16" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J43" s="20" t="s">
         <v>19</v>
@@ -3950,7 +3950,7 @@
     </row>
     <row r="44" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B44" s="15">
         <v>10</v>
@@ -3964,10 +3964,10 @@
         <v/>
       </c>
       <c r="E44" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G44" s="15" t="s">
         <v>34</v>
@@ -3976,7 +3976,7 @@
         <v>22</v>
       </c>
       <c r="I44" s="16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J44" s="20" t="s">
         <v>19</v>
@@ -3988,7 +3988,7 @@
     </row>
     <row r="45" spans="1:12" ht="182" x14ac:dyDescent="0.2">
       <c r="A45" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B45" s="15">
         <v>10</v>
@@ -4002,10 +4002,10 @@
         <v/>
       </c>
       <c r="E45" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G45" s="15" t="s">
         <v>22</v>
@@ -4014,7 +4014,7 @@
         <v>28</v>
       </c>
       <c r="I45" s="16" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J45" s="20" t="s">
         <v>30</v>
@@ -4023,12 +4023,12 @@
         <v>1</v>
       </c>
       <c r="L45" s="22" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A46" s="15" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B46" s="15">
         <v>10</v>
@@ -4042,10 +4042,10 @@
         <v/>
       </c>
       <c r="E46" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F46" s="16" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G46" s="15" t="s">
         <v>28</v>
@@ -4054,7 +4054,7 @@
         <v>34</v>
       </c>
       <c r="I46" s="16" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J46" s="20" t="s">
         <v>19</v>
@@ -4066,7 +4066,7 @@
     </row>
     <row r="47" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B47" s="15">
         <v>10</v>
@@ -4080,10 +4080,10 @@
         <v/>
       </c>
       <c r="E47" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F47" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G47" s="15" t="s">
         <v>28</v>
@@ -4092,7 +4092,7 @@
         <v>17</v>
       </c>
       <c r="I47" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J47" s="20" t="s">
         <v>19</v>
@@ -4104,7 +4104,7 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" s="15" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B48" s="15">
         <v>10</v>
@@ -4118,10 +4118,10 @@
         <v/>
       </c>
       <c r="E48" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F48" s="16" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G48" s="15" t="s">
         <v>28</v>
@@ -4130,7 +4130,7 @@
         <v>34</v>
       </c>
       <c r="I48" s="16" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J48" s="20" t="s">
         <v>19</v>
@@ -4142,7 +4142,7 @@
     </row>
     <row r="49" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="15" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B49" s="15">
         <v>10</v>
@@ -4156,10 +4156,10 @@
         <v/>
       </c>
       <c r="E49" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F49" s="16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G49" s="15" t="s">
         <v>28</v>
@@ -4168,7 +4168,7 @@
         <v>22</v>
       </c>
       <c r="I49" s="16" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J49" s="20" t="s">
         <v>19</v>
@@ -4180,7 +4180,7 @@
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A50" s="15" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B50" s="15">
         <v>10</v>
@@ -4194,10 +4194,10 @@
         <v/>
       </c>
       <c r="E50" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F50" s="16" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G50" s="15" t="s">
         <v>22</v>
@@ -4206,7 +4206,7 @@
         <v>17</v>
       </c>
       <c r="I50" s="16" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J50" s="20" t="s">
         <v>19</v>
@@ -4218,7 +4218,7 @@
     </row>
     <row r="51" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="17" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B51" s="17">
         <v>11</v>
@@ -4232,10 +4232,10 @@
         <v/>
       </c>
       <c r="E51" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="F51" s="18" t="s">
         <v>180</v>
-      </c>
-      <c r="F51" s="18" t="s">
-        <v>181</v>
       </c>
       <c r="G51" s="17" t="s">
         <v>22</v>
@@ -4244,7 +4244,7 @@
         <v>34</v>
       </c>
       <c r="I51" s="18" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J51" s="20" t="s">
         <v>19</v>
@@ -4256,7 +4256,7 @@
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A52" s="17" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B52" s="17">
         <v>11</v>
@@ -4270,10 +4270,10 @@
         <v/>
       </c>
       <c r="E52" s="17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F52" s="18" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G52" s="17" t="s">
         <v>34</v>
@@ -4282,7 +4282,7 @@
         <v>22</v>
       </c>
       <c r="I52" s="18" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J52" s="20" t="s">
         <v>19</v>
@@ -4294,7 +4294,7 @@
     </row>
     <row r="53" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B53" s="17">
         <v>11</v>
@@ -4308,10 +4308,10 @@
         <v/>
       </c>
       <c r="E53" s="17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F53" s="18" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G53" s="17" t="s">
         <v>22</v>
@@ -4320,7 +4320,7 @@
         <v>28</v>
       </c>
       <c r="I53" s="18" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="J53" s="20" t="s">
         <v>19</v>
@@ -4332,7 +4332,7 @@
     </row>
     <row r="54" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="17" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B54" s="17">
         <v>11</v>
@@ -4346,10 +4346,10 @@
         <v/>
       </c>
       <c r="E54" s="17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F54" s="18" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G54" s="17" t="s">
         <v>28</v>
@@ -4358,7 +4358,7 @@
         <v>34</v>
       </c>
       <c r="I54" s="18" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J54" s="20" t="s">
         <v>19</v>
@@ -4370,7 +4370,7 @@
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A55" s="17" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B55" s="17">
         <v>11</v>
@@ -4384,10 +4384,10 @@
         <v/>
       </c>
       <c r="E55" s="17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F55" s="18" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G55" s="17" t="s">
         <v>22</v>
@@ -4396,7 +4396,7 @@
         <v>17</v>
       </c>
       <c r="I55" s="18" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="J55" s="20" t="s">
         <v>19</v>
@@ -4408,7 +4408,7 @@
     </row>
     <row r="56" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="17" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B56" s="17">
         <v>12</v>
@@ -4422,10 +4422,10 @@
         <v/>
       </c>
       <c r="E56" s="17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F56" s="18" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G56" s="17" t="s">
         <v>22</v>
@@ -4434,7 +4434,7 @@
         <v>17</v>
       </c>
       <c r="I56" s="18" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="J56" s="20" t="s">
         <v>19</v>
@@ -4446,7 +4446,7 @@
     </row>
     <row r="57" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="17" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B57" s="17">
         <v>12</v>
@@ -4460,10 +4460,10 @@
         <v/>
       </c>
       <c r="E57" s="17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F57" s="18" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G57" s="17" t="s">
         <v>17</v>
@@ -4472,7 +4472,7 @@
         <v>17</v>
       </c>
       <c r="I57" s="18" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J57" s="20" t="s">
         <v>19</v>
@@ -4484,7 +4484,7 @@
     </row>
     <row r="58" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="17" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B58" s="17">
         <v>12</v>
@@ -4498,10 +4498,10 @@
         <v/>
       </c>
       <c r="E58" s="17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F58" s="18" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G58" s="17" t="s">
         <v>34</v>
@@ -4510,7 +4510,7 @@
         <v>17</v>
       </c>
       <c r="I58" s="18" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="J58" s="20" t="s">
         <v>19</v>
@@ -4522,7 +4522,7 @@
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A59" s="17" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B59" s="17">
         <v>12</v>
@@ -4536,10 +4536,10 @@
         <v/>
       </c>
       <c r="E59" s="17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F59" s="18" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G59" s="17" t="s">
         <v>17</v>
@@ -4548,7 +4548,7 @@
         <v>17</v>
       </c>
       <c r="I59" s="18" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="J59" s="20" t="s">
         <v>19</v>
@@ -4614,138 +4614,138 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>283</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="55" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="27" t="s">
+        <v>284</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>285</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="C5" s="8" t="s">
         <v>286</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="D5" s="8" t="s">
         <v>287</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="27" t="s">
+        <v>288</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>289</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="C6" s="8" t="s">
         <v>290</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="D6" s="8" t="s">
         <v>291</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="70" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="27" t="s">
+        <v>292</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>293</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="C7" s="8" t="s">
         <v>294</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="D7" s="8" t="s">
         <v>295</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="40" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="27" t="s">
+        <v>296</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>297</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C8" s="8" t="s">
         <v>298</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="D8" s="8" t="s">
         <v>299</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="27" t="s">
+        <v>300</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>301</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="C9" s="8" t="s">
         <v>302</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="D9" s="8" t="s">
         <v>303</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="70" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="27" t="s">
+        <v>304</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>305</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="C10" s="8" t="s">
         <v>306</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="D10" s="8" t="s">
         <v>307</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="27" t="s">
+        <v>308</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>309</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="C11" s="8" t="s">
         <v>310</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="D11" s="8" t="s">
         <v>311</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="27" t="s">
+        <v>312</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>313</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="C12" s="8" t="s">
         <v>314</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="D12" s="8" t="s">
         <v>315</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>316</v>
       </c>
     </row>
   </sheetData>
@@ -4770,32 +4770,32 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>323</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>324</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>11</v>
@@ -4803,19 +4803,19 @@
     </row>
     <row r="5" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="B5" s="8" t="s">
         <v>325</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>326</v>
       </c>
       <c r="C5" s="7" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="8" t="s">
+        <v>326</v>
+      </c>
+      <c r="E5" s="7" t="s">
         <v>327</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>328</v>
       </c>
       <c r="F5" s="7">
         <v>12</v>
@@ -4826,19 +4826,19 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>329</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>330</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F6" s="7">
         <v>2</v>
@@ -4849,10 +4849,10 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>331</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>332</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>22</v>
@@ -4861,7 +4861,7 @@
         <v>34</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F7" s="7">
         <v>2</v>
@@ -4872,19 +4872,19 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>333</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>334</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F8" s="7">
         <v>2</v>
@@ -4895,19 +4895,19 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>336</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>337</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>34</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F9" s="7">
         <v>4</v>
@@ -4918,19 +4918,19 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>338</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>339</v>
       </c>
       <c r="C10" s="7" t="s">
         <v>34</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F10" s="7">
         <v>4</v>
@@ -4941,19 +4941,19 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
+        <v>340</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>341</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>342</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>34</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F11" s="7">
         <v>8</v>
@@ -4964,19 +4964,19 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>343</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>344</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F12" s="7">
         <v>8</v>
@@ -4987,19 +4987,19 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
+        <v>344</v>
+      </c>
+      <c r="B13" s="8" t="s">
         <v>345</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>346</v>
       </c>
       <c r="C13" s="7" t="s">
         <v>34</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F13" s="7">
         <v>8</v>
@@ -5010,19 +5010,19 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>348</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>349</v>
       </c>
       <c r="C14" s="7" t="s">
         <v>34</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F14" s="7">
         <v>10</v>
@@ -5033,19 +5033,19 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>350</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>351</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F15" s="7">
         <v>10</v>
@@ -5056,19 +5056,19 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="B16" s="8" t="s">
         <v>353</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>354</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F16" s="7">
         <v>10</v>
@@ -5079,10 +5079,10 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
+        <v>355</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>356</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>357</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>28</v>
@@ -5091,7 +5091,7 @@
         <v>22</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F17" s="7">
         <v>10</v>
@@ -5102,19 +5102,19 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>358</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>359</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>22</v>
       </c>
       <c r="D18" s="8" t="s">
+        <v>359</v>
+      </c>
+      <c r="E18" s="7" t="s">
         <v>360</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>361</v>
       </c>
       <c r="F18" s="7">
         <v>12</v>
@@ -5125,19 +5125,19 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="B19" s="8" t="s">
         <v>362</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>363</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>22</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F19" s="7">
         <v>11</v>
@@ -5173,12 +5173,12 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -5186,22 +5186,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>367</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>368</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>370</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.2">
@@ -5213,16 +5213,16 @@
         <v>34</v>
       </c>
       <c r="D5" s="30" t="s">
+        <v>371</v>
+      </c>
+      <c r="E5" s="30" t="s">
         <v>372</v>
       </c>
-      <c r="E5" s="30" t="s">
+      <c r="F5" s="30" t="s">
         <v>373</v>
       </c>
-      <c r="F5" s="30" t="s">
+      <c r="G5" s="30" t="s">
         <v>374</v>
-      </c>
-      <c r="G5" s="30" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="98" customHeight="1" x14ac:dyDescent="0.2">
@@ -5236,16 +5236,16 @@
         <v>22</v>
       </c>
       <c r="D6" s="22" t="s">
+        <v>375</v>
+      </c>
+      <c r="E6" s="22" t="s">
         <v>376</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="F6" s="22" t="s">
         <v>377</v>
       </c>
-      <c r="F6" s="22" t="s">
+      <c r="G6" s="22" t="s">
         <v>378</v>
-      </c>
-      <c r="G6" s="22" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="98" customHeight="1" x14ac:dyDescent="0.2">
@@ -5259,16 +5259,16 @@
         <v>22</v>
       </c>
       <c r="D7" s="22" t="s">
+        <v>379</v>
+      </c>
+      <c r="E7" s="22" t="s">
         <v>380</v>
       </c>
-      <c r="E7" s="22" t="s">
+      <c r="F7" s="22" t="s">
         <v>381</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="G7" s="22" t="s">
         <v>382</v>
-      </c>
-      <c r="G7" s="22" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="210" x14ac:dyDescent="0.2">
@@ -5282,16 +5282,16 @@
         <v>22</v>
       </c>
       <c r="D8" s="22" t="s">
+        <v>383</v>
+      </c>
+      <c r="E8" s="22" t="s">
         <v>384</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="F8" s="22" t="s">
         <v>385</v>
       </c>
-      <c r="F8" s="22" t="s">
+      <c r="G8" s="22" t="s">
         <v>386</v>
-      </c>
-      <c r="G8" s="22" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="306" x14ac:dyDescent="0.2">
@@ -5305,16 +5305,16 @@
         <v>22</v>
       </c>
       <c r="D9" s="22" t="s">
+        <v>407</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>401</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>405</v>
+      </c>
+      <c r="G9" s="22" t="s">
         <v>408</v>
-      </c>
-      <c r="E9" s="22" t="s">
-        <v>402</v>
-      </c>
-      <c r="F9" s="22" t="s">
-        <v>406</v>
-      </c>
-      <c r="G9" s="22" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -6108,20 +6108,20 @@
   <sheetData>
     <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>30</v>
@@ -6130,16 +6130,16 @@
         <v>24</v>
       </c>
       <c r="E4" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>391</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>392</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>393</v>
-      </c>
-      <c r="H4" s="6" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -6152,11 +6152,11 @@
       </c>
       <c r="C5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Hoàn thành")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Đang làm")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Trễ hạn")</f>
@@ -6164,11 +6164,11 @@
       </c>
       <c r="F5" s="34">
         <f>IFERROR(C5/B5,0)</f>
-        <v>0.57894736842105265</v>
+        <v>0.63157894736842102</v>
       </c>
       <c r="G5" s="34">
         <f>IFERROR(AVERAGEIF('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.66842105263157892</v>
+        <v>0.67368421052631577</v>
       </c>
       <c r="H5" s="7">
         <f>COUNTIF('Kế hoạch'!$H$5:$H$109,A5)</f>
@@ -6276,7 +6276,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="27" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B9" s="35">
         <f>SUM(B5:B8)</f>
@@ -6284,11 +6284,11 @@
       </c>
       <c r="C9" s="35">
         <f>SUM(C5:C8)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D9" s="35">
         <f>SUM(D5:D8)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E9" s="35">
         <f>SUM(E5:E8)</f>
@@ -6296,11 +6296,11 @@
       </c>
       <c r="F9" s="36">
         <f>IFERROR(C9/B9,0)</f>
-        <v>0.36363636363636365</v>
+        <v>0.38181818181818183</v>
       </c>
       <c r="G9" s="36">
         <f>IFERROR(AVERAGE('Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.40000000000000008</v>
+        <v>0.40181818181818185</v>
       </c>
       <c r="H9" s="35">
         <f>SUM(H5:H8)</f>
@@ -6309,7 +6309,7 @@
     </row>
     <row r="12" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
@@ -6317,7 +6317,7 @@
         <v>6</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>30</v>
@@ -6353,16 +6353,16 @@
       </c>
       <c r="C15" s="11">
         <f>COUNTIFS('Kế hoạch'!$E$5:$E$109,A15,'Kế hoạch'!$J$5:$J$109,"Hoàn thành")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D15" s="38">
         <f>IFERROR(C15/B15,0)</f>
-        <v>0.8571428571428571</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="13" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B16" s="13">
         <f>COUNTIF('Kế hoạch'!$E$5:$E$109,A16)</f>
@@ -6379,7 +6379,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B17" s="15">
         <f>COUNTIF('Kế hoạch'!$E$5:$E$109,A17)</f>
@@ -6396,7 +6396,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B18" s="17">
         <f>COUNTIF('Kế hoạch'!$E$5:$E$109,A18)</f>
@@ -6413,7 +6413,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
T31: nháp báo cáo v2.2 – phần mảng B mục 2.2, 2.3, 3; cập nhật mục 1, 2.1; kế hoạch
Báo cáo đổi tên _v2.1 → _v2.2 (bản v2.1 đã nộp còn trong lịch sử git).
- 2.2: bước ánh xạ, 8C cho LICH_HEN, lược đồ quan hệ, khóa ngoại mảng B
- 2.3: FD, khóa ứng viên, chứng minh BCNF mảng B
- 3: từ điển dữ liệu 4 bảng, miền giá trị dùng chung
- Phần A, C để chữ xám chờ T19, T21, T23, T25, T26, T28, T29
- Mục 1, 2.1: bối cảnh một cơ sở, không đặt lịch trực tuyến; phạm vi có tài
  khoản; tác nhân lễ tân, bác sĩ theo BR-B08, B10; thuật ngữ tái khám;
  2.1.5 BR-B03; 2.1.6 quyết định giấy chuyển, trạng thái lịch hẹn
- Giãn dòng 1.2, cách đoạn 3pt; tách hình và chú thích khỏi nội dung
B_schema.sql: CHECK email, ngày sinh theo ràng buộc chung 1.2.4 (L06 ở T30).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khoile/Documents/PTIT/HK5/CSDL/telemedicine/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABCFF4B7-E797-124B-BDC6-E0973C12BA8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A090BDD-7F7F-7E45-AA7B-371E0D03CF25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1200" yWindow="660" windowWidth="29040" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="410">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="411">
   <si>
     <t>Kế hoạch công việc theo tuần</t>
   </si>
@@ -1334,15 +1334,13 @@
     <t>docs/6_chuan-hoa/T30_ReviewCheo.md – đã rà phần B (Khôi, 27/10): L01 sửa T20 (FK kép giấy – bệnh nhân); L02–L04 diễn giải trigger đã xác nhận, ghi vào T08 mục 5; ERD B không phải sửa; chờ A, C (T19, T21, T26, T28), mục 3 (T29); C1 vai_tro/loai_nv chờ nhóm họp</t>
   </si>
   <si>
-    <t>Hữu Khoa: chốt phương án ánh xạ BAC_SI (8A hay 8C) ở T19 – ảnh hưởng FK ma_bac_si_lap → BAC_SI_DA_KHOA; review T20
-Đăng Khoa: review T24; chốt cách trình bày FD có điều kiện ở T22
-Đăng Khoa: review T27; T30 chốt TAI_KHOAN.vai_tro (giữ hay suy từ loai_nv)
-Hữu Khoa: T18 chốt kiểu khóa (INTEGER identity), giá trị loai_nv trùng vai_tro (QUAN_TRI_NHAN_SU, QUAN_TRI_TAI_KHOAN, QUAN_TRI_DANH_MUC, BAC_SI, LE_TAN); review T33
-Đăng Khoa: review T37; T39 seed phải thêm lịch hẹn ở DA_DAT rồi UPDATE, lịch nằm trong ca, lịch chuyên khoa có giấy hoặc tái khám
-Cả nhóm: họp chốt C1 (TAI_KHOAN.vai_tro trùng loai_nv, BR-B10 đổi vai trò mâu thuẫn BR-A09)</t>
-  </si>
-  <si>
     <t>sql/queries_B.sql – Q1 tỷ lệ hủy/vắng theo bác sĩ (JOIN, FILTER, HAVING); Q2 doanh thu chuyên khoa theo tháng (hàm cửa sổ); Q3 bệnh nhân &gt; 3 lần khám/6 tháng (subquery FROM + EXISTS tương quan); Q4 khung giờ đông nhất, tỷ lệ từ xa (ROLLUP, RANK). Kiểm chứng trên dữ liệu thử qua trigger, đối chiếu tính độc lập bằng Python: khớp (27/10). Chờ Đăng Khoa review</t>
+  </si>
+  <si>
+    <t>docs/INT1313_TX_G5_DeTai05_Telemedicine_v2.1.docx – mục Giới thiệu tóm tắt, 1, 1.2, 2, 2.1 hoàn chỉnh, có ERD tổng; đã nộp 21/10/2026</t>
+  </si>
+  <si>
+    <t>docs/INT1313_TX_G5_DeTai05_Telemedicine_v2.2.docx (nháp, 27/10) – trang bìa v2.2; đã điền phần B mục 2.2 (bước ánh xạ, 8C cho LICH_HEN, lược đồ, khóa ngoại), 2.3 (FD, khóa, chứng minh BCNF), 3 (4 bảng, miền giá trị); phần A, C để chữ xám chờ T19, T21, T23, T25, T26, T28, T29; còn Hình 2.2, review chéo, nộp</t>
   </si>
   <si>
     <t>T20: ánh xạ mảng B sang lược đồ quan hệ (Elmasri bước 1–8): 4 bảng, PK/FK, UNIQUE; phân lớp LICH_HEN chọn 8C; truy vết ERD → lược đồ, quy tắc còn lại cho cài đặt
@@ -1351,7 +1349,17 @@
 T33 (làm sớm): DDL mảng B, chạy thử 17 ca vi phạm trên PG16 đều bị chặn
 T37 (làm sớm): 4 trigger + view v_lich_hen_hom_nay mảng B, chạy thử 17 ca vi phạm đều bị chặn
 T30 (phần B): đối chiếu T20, T24, T27 với DDL, trigger; sửa T20 (FK kép giấy – bệnh nhân); lập danh sách lỗi, bảng quy tắc → cơ chế
-T41 (làm sớm): 4 truy vấn mảng B, kiểm chứng trên dữ liệu thử đi qua trigger</t>
+T41 (làm sớm): 4 truy vấn mảng B, kiểm chứng trên dữ liệu thử đi qua trigger
+T31 (nháp v2.2): điền phần B mục 2.2, 2.3, 3 vào báo cáo (đổi tên file sang _v2.2); bổ sung CHECK email, ngày sinh cho benh_nhan theo 1.2.4</t>
+  </si>
+  <si>
+    <t>Hữu Khoa: chốt phương án ánh xạ BAC_SI (8A hay 8C) ở T19 – ảnh hưởng FK ma_bac_si_lap → BAC_SI_DA_KHOA; review T20
+Đăng Khoa: review T24; chốt cách trình bày FD có điều kiện ở T22
+Đăng Khoa: review T27; T30 chốt TAI_KHOAN.vai_tro (giữ hay suy từ loai_nv)
+Hữu Khoa: T18 chốt kiểu khóa (INTEGER identity), giá trị loai_nv trùng vai_tro (QUAN_TRI_NHAN_SU, QUAN_TRI_TAI_KHOAN, QUAN_TRI_DANH_MUC, BAC_SI, LE_TAN); review T33
+Đăng Khoa: review T37; T39 seed phải thêm lịch hẹn ở DA_DAT rồi UPDATE, lịch nằm trong ca, lịch chuyên khoa có giấy hoặc tái khám
+Cả nhóm: họp chốt C1 (TAI_KHOAN.vai_tro trùng loai_nv, BR-B10 đổi vai trò mâu thuẫn BR-A09)
+Hữu Khoa, Đăng Khoa: điền phần A, C vào docs/…_v2.2.docx (chỗ chữ xám); Hữu Khoa vẽ Hình 2.2 lược đồ quan hệ</t>
   </si>
   <si>
     <t>docs/5_anh-xa/T20_AnhXa_MangB.md
@@ -1361,10 +1369,8 @@
 sql/B_schema.sql
 sql/B_trigger_view.sql
 docs/6_chuan-hoa/T30_ReviewCheo.md
-sql/queries_B.sql</t>
-  </si>
-  <si>
-    <t>docs/INT1313_TX_G5_DeTai05_Telemedicine_v2.1.docx – mục Giới thiệu tóm tắt, 1, 1.2, 2, 2.1 hoàn chỉnh, có ERD tổng; đã nộp 21/10/2026</t>
+sql/queries_B.sql
+docs/INT1313_TX_G5_DeTai05_Telemedicine_v2.2.docx</t>
   </si>
 </sst>
 </file>
@@ -3097,7 +3103,7 @@
         <v>1</v>
       </c>
       <c r="L21" s="22" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
@@ -3602,7 +3608,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:12" ht="154" x14ac:dyDescent="0.2">
       <c r="A35" s="13" t="s">
         <v>129</v>
       </c>
@@ -3633,12 +3639,14 @@
         <v>131</v>
       </c>
       <c r="J35" s="20" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="K35" s="21">
-        <v>0</v>
-      </c>
-      <c r="L35" s="22"/>
+        <v>0.3</v>
+      </c>
+      <c r="L35" s="22" t="s">
+        <v>407</v>
+      </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="15" t="s">
@@ -4023,7 +4031,7 @@
         <v>1</v>
       </c>
       <c r="L45" s="22" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.2">
@@ -5005,7 +5013,7 @@
         <v>8</v>
       </c>
       <c r="G13" s="20" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -5294,7 +5302,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="306" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="345" x14ac:dyDescent="0.2">
       <c r="A9" s="20">
         <v>4</v>
       </c>
@@ -5305,16 +5313,16 @@
         <v>22</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="E9" s="22" t="s">
         <v>401</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -6156,7 +6164,7 @@
       </c>
       <c r="D5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Đang làm")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Trễ hạn")</f>
@@ -6168,7 +6176,7 @@
       </c>
       <c r="G5" s="34">
         <f>IFERROR(AVERAGEIF('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.67368421052631577</v>
+        <v>0.68947368421052635</v>
       </c>
       <c r="H5" s="7">
         <f>COUNTIF('Kế hoạch'!$H$5:$H$109,A5)</f>
@@ -6288,7 +6296,7 @@
       </c>
       <c r="D9" s="35">
         <f>SUM(D5:D8)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9" s="35">
         <f>SUM(E5:E8)</f>
@@ -6300,7 +6308,7 @@
       </c>
       <c r="G9" s="36">
         <f>IFERROR(AVERAGE('Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.40181818181818185</v>
+        <v>0.40727272727272729</v>
       </c>
       <c r="H9" s="35">
         <f>SUM(H5:H8)</f>

</xml_diff>

<commit_message>
T46, T43: phần mảng B mục 4.1, 4.2, 5.1 trong báo cáo; sql/tests_B.sql; kế hoạch
- sql/tests_B.sql: 49 ca tự kiểm (38 phải bị từ chối, 10 hợp lệ, 1 view),
  ROLLBACK cuối; 49/49 đạt trên PG16 (CSDL trống và CSDL có ~600 lịch hẹn),
  bảng mảng A giả lập
- Báo cáo: 4.1.1 trích DDL lich_hen, kiểu dữ liệu; 4.1.2 chỉ mục; 4.1.3
  v_lich_hen_hom_nay; 4.1.4 5 trigger; 4.1.6 cơ chế BR-B03, B04, B06, B07,
  B09, B10 theo cài đặt thực tế; 4.2.1–4.2.2 Q05–Q08; 5.1 18 ca tiêu biểu
- queries_B.sql: đánh số Q05–Q08 theo báo cáo, gói dòng ≤ 80 ký tự; đối
  chiếu lại với tính độc lập: khớp

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/khoile/Documents/PTIT/HK5/CSDL/telemedicine/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A090BDD-7F7F-7E45-AA7B-371E0D03CF25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47822B3B-2B28-D144-97C3-33F4A05590AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1200" yWindow="660" windowWidth="29040" windowHeight="18980" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="705" uniqueCount="413">
   <si>
     <t>Kế hoạch công việc theo tuần</t>
   </si>
@@ -1343,6 +1343,12 @@
     <t>docs/INT1313_TX_G5_DeTai05_Telemedicine_v2.2.docx (nháp, 27/10) – trang bìa v2.2; đã điền phần B mục 2.2 (bước ánh xạ, 8C cho LICH_HEN, lược đồ, khóa ngoại), 2.3 (FD, khóa, chứng minh BCNF), 3 (4 bảng, miền giá trị); phần A, C để chữ xám chờ T19, T21, T23, T25, T26, T28, T29; còn Hình 2.2, review chéo, nộp</t>
   </si>
   <si>
+    <t>Phần B đã vào docs/…_v2.2.docx (27/10): 4.1.1 trích DDL lich_hen + kiểu dữ liệu; 4.1.2 chỉ mục; 4.1.3 v_lich_hen_hom_nay; 4.1.4 5 trigger; 4.1.6 sửa cơ chế BR-B03, B04, B06, B07, B09, B10 theo cài đặt; 4.2.1–4.2.2 Q05–Q08 (yêu cầu, SQL, cách hoạt động); 5.1 18 ca tiêu biểu từ tests_B.sql. Chờ A, C (T32, T34, T36, T38, T40, T42), seed T39 (kết quả mẫu), T44 hiệu năng, T45 RBAC; nộp v3</t>
+  </si>
+  <si>
+    <t>Phần B: sql/tests_B.sql – 49 ca tự kiểm (38 bị từ chối, 10 hợp lệ, 1 view), ROLLBACK cuối; 49/49 đạt trên PG16 với bảng A giả lập (27/10). Đăng Khoa gộp vào tests.sql</t>
+  </si>
+  <si>
     <t>T20: ánh xạ mảng B sang lược đồ quan hệ (Elmasri bước 1–8): 4 bảng, PK/FK, UNIQUE; phân lớp LICH_HEN chọn 8C; truy vết ERD → lược đồ, quy tắc còn lại cho cài đặt
 T24: FD và khóa ứng viên 4 bảng mảng B, ghi FD đã xét và loại; nêu 2 điểm cho T27/T30 (FD có điều kiện trên cột UNIQUE cho phép NULL; TAI_KHOAN.vai_tro trùng NHAN_VIEN.loai_nv)
 T27: chứng minh 1NF → BCNF 4 bảng mảng B, không phải tách; ghi các thiết kế đã tránh vi phạm 3NF
@@ -1350,7 +1356,8 @@
 T37 (làm sớm): 4 trigger + view v_lich_hen_hom_nay mảng B, chạy thử 17 ca vi phạm đều bị chặn
 T30 (phần B): đối chiếu T20, T24, T27 với DDL, trigger; sửa T20 (FK kép giấy – bệnh nhân); lập danh sách lỗi, bảng quy tắc → cơ chế
 T41 (làm sớm): 4 truy vấn mảng B, kiểm chứng trên dữ liệu thử đi qua trigger
-T31 (nháp v2.2): điền phần B mục 2.2, 2.3, 3 vào báo cáo (đổi tên file sang _v2.2); bổ sung CHECK email, ngày sinh cho benh_nhan theo 1.2.4</t>
+T31 (nháp v2.2): điền phần B mục 2.2, 2.3, 3 vào báo cáo (đổi tên file sang _v2.2); bổ sung CHECK email, ngày sinh cho benh_nhan theo 1.2.4
+T46 (phần B): điền mục 4.1, 4.2, 5.1 phần B vào báo cáo; T43 (phần B): sql/tests_B.sql 49/49 đạt; Q05–Q08 gói dòng ≤ 80 ký tự, đối chiếu lại khớp</t>
   </si>
   <si>
     <t>Hữu Khoa: chốt phương án ánh xạ BAC_SI (8A hay 8C) ở T19 – ảnh hưởng FK ma_bac_si_lap → BAC_SI_DA_KHOA; review T20
@@ -1359,7 +1366,8 @@
 Hữu Khoa: T18 chốt kiểu khóa (INTEGER identity), giá trị loai_nv trùng vai_tro (QUAN_TRI_NHAN_SU, QUAN_TRI_TAI_KHOAN, QUAN_TRI_DANH_MUC, BAC_SI, LE_TAN); review T33
 Đăng Khoa: review T37; T39 seed phải thêm lịch hẹn ở DA_DAT rồi UPDATE, lịch nằm trong ca, lịch chuyên khoa có giấy hoặc tái khám
 Cả nhóm: họp chốt C1 (TAI_KHOAN.vai_tro trùng loai_nv, BR-B10 đổi vai trò mâu thuẫn BR-A09)
-Hữu Khoa, Đăng Khoa: điền phần A, C vào docs/…_v2.2.docx (chỗ chữ xám); Hữu Khoa vẽ Hình 2.2 lược đồ quan hệ</t>
+Hữu Khoa, Đăng Khoa: điền phần A, C vào docs/…_v2.2.docx (chỗ chữ xám); Hữu Khoa vẽ Hình 2.2 lược đồ quan hệ
+Đăng Khoa: gộp tests_B.sql vào tests.sql (T43); T39 seed để có kết quả mẫu Q05–Q08</t>
   </si>
   <si>
     <t>docs/5_anh-xa/T20_AnhXa_MangB.md
@@ -1370,7 +1378,8 @@
 sql/B_trigger_view.sql
 docs/6_chuan-hoa/T30_ReviewCheo.md
 sql/queries_B.sql
-docs/INT1313_TX_G5_DeTai05_Telemedicine_v2.2.docx</t>
+docs/INT1313_TX_G5_DeTai05_Telemedicine_v2.2.docx
+sql/tests_B.sql</t>
   </si>
 </sst>
 </file>
@@ -4108,7 +4117,9 @@
       <c r="K47" s="21">
         <v>0</v>
       </c>
-      <c r="L47" s="22"/>
+      <c r="L47" s="22" t="s">
+        <v>409</v>
+      </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" s="15" t="s">
@@ -4186,7 +4197,7 @@
       </c>
       <c r="L49" s="22"/>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:12" ht="196" x14ac:dyDescent="0.2">
       <c r="A50" s="15" t="s">
         <v>175</v>
       </c>
@@ -4217,12 +4228,14 @@
         <v>177</v>
       </c>
       <c r="J50" s="20" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="K50" s="21">
-        <v>0</v>
-      </c>
-      <c r="L50" s="22"/>
+        <v>0.3</v>
+      </c>
+      <c r="L50" s="22" t="s">
+        <v>408</v>
+      </c>
     </row>
     <row r="51" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="17" t="s">
@@ -5036,7 +5049,7 @@
         <v>10</v>
       </c>
       <c r="G14" s="20" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -5059,7 +5072,7 @@
         <v>10</v>
       </c>
       <c r="G15" s="20" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -5082,7 +5095,7 @@
         <v>10</v>
       </c>
       <c r="G16" s="20" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
@@ -5302,7 +5315,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="345" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="384" x14ac:dyDescent="0.2">
       <c r="A9" s="20">
         <v>4</v>
       </c>
@@ -5313,16 +5326,16 @@
         <v>22</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="E9" s="22" t="s">
         <v>401</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -6164,7 +6177,7 @@
       </c>
       <c r="D5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Đang làm")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" s="7">
         <f>COUNTIFS('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$J$5:$J$109,"Trễ hạn")</f>
@@ -6176,7 +6189,7 @@
       </c>
       <c r="G5" s="34">
         <f>IFERROR(AVERAGEIF('Kế hoạch'!$G$5:$G$109,A5,'Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.68947368421052635</v>
+        <v>0.70526315789473693</v>
       </c>
       <c r="H5" s="7">
         <f>COUNTIF('Kế hoạch'!$H$5:$H$109,A5)</f>
@@ -6296,7 +6309,7 @@
       </c>
       <c r="D9" s="35">
         <f>SUM(D5:D8)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E9" s="35">
         <f>SUM(E5:E8)</f>
@@ -6308,7 +6321,7 @@
       </c>
       <c r="G9" s="36">
         <f>IFERROR(AVERAGE('Kế hoạch'!$K$5:$K$109),0)</f>
-        <v>0.40727272727272729</v>
+        <v>0.41272727272727278</v>
       </c>
       <c r="H9" s="35">
         <f>SUM(H5:H8)</f>

</xml_diff>

<commit_message>
T29: từ điển dữ liệu mục 3 đủ A, B, C; sửa bảng A lệch cột; cập nhật T30, kế hoạch
- Báo cáo v2.2 mục 3: danh sách 19 bảng theo A, B, C; thêm 9 bảng C theo C_schema.sql,
  C_trigger_view.sql; viết lại 6 bảng A cùng khuôn B (cột lệch, tiêu đề Heading 3);
  bảng miền giá trị thêm trang_thai_ho_so, bỏ dòng chờ.
- T30: L07 (bảng A lệch cột, đã sửa), L08 (T25 và DDL lệch về ten_hoat_chat UNIQUE, chờ sửa).
- Kế hoạch: T29 hoàn thành; cập nhật T30, T31; mục 3 sheet Viết báo cáo hoàn thành.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -2913,15 +2913,15 @@
       </c>
       <c r="J33" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="K33" s="21" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="L33" s="22" t="inlineStr">
         <is>
-          <t>Phần A: docs/6_chuan-hoa/T29_TuDienDuLieu_MangA.md, đã vào báo cáo v2.2 mục 3 (6 bảng); phần B đã có trong báo cáo (Khôi, T31). Còn: bảng mảng C (Đăng Khoa), bảng miền giá trị phần A, C; Hữu Khoa gộp</t>
+          <t>Báo cáo v2.2 mục 3 (28/10, Khôi gộp): danh sách 19 bảng A, B, C; mô tả chi tiết từng bảng cùng khuôn (Kiểu, Null, Khóa, Mặc định, Ràng buộc kèm BR, Mô tả) theo A/B/C_schema.sql và trigger; 9 miền giá trị (thêm trang_thai_ho_so). Viết lại 6 bảng A bị lệch cột (T30 L07); nguồn A: docs/6_chuan-hoa/T29_TuDienDuLieu_MangA.md. Chờ Hữu Khoa, Đăng Khoa xác nhận phần mình</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="L34" s="22" t="inlineStr">
         <is>
-          <t>docs/6_chuan-hoa/T30_ReviewCheo.md – B: Khôi tự rà (L01–L06 đã sửa), Đăng Khoa review chéo 28/10, tests_B 49/49 trên A stub. A (T19, T23, T26, T29), C (T21, T25, T28) đủ tài liệu, chờ review chéo độc lập; C tự rà ở mục 8 (ham_luong, created_by trên ERD C). C2, C3 đã chốt; C1 vai_tro/loai_nv chờ họp</t>
+          <t>docs/6_chuan-hoa/T30_ReviewCheo.md – B: Khôi tự rà (L01–L06 đã sửa), Đăng Khoa review chéo 28/10, tests_B 49/49 trên A stub. Mục 3: L07 bảng A lệch cột (đã sửa), L08 T25 ghi tên hoạt chất không duy nhất nhưng DDL UNIQUE (chờ Đăng Khoa). A (T19, T23, T26), C (T21, T25, T28) đủ tài liệu, chờ review chéo độc lập; C tự rà ở mục 8. C2, C3 đã chốt; C1 vai_tro/loai_nv chờ họp</t>
         </is>
       </c>
     </row>
@@ -3029,11 +3029,11 @@
         </is>
       </c>
       <c r="K35" s="21" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="L35" s="22" t="inlineStr">
         <is>
-          <t>docs/INT1313_TX_G5_DeTai05_Telemedicine_v2.2.docx (nháp) – phần B đã điền 2.2, 2.3, 3 (27/10). Phần A đã có 2.2.3 (lý do 8A), 2.3.3, mục 3 (6 bảng). Còn chữ xám: 2.2.2, 2.2.4, 2.2.5 phần A, C; 2.3.3 phần C; mục 3 bảng C và miền giá trị A, C; Hình 2.2; review chéo T30, nộp</t>
+          <t>docs/INT1313_TX_G5_DeTai05_Telemedicine_v2.2.docx (nháp) – phần B đã điền 2.2, 2.3, 3 (27/10). Phần A đã có 2.2.3 (lý do 8A), 2.3.3. Mục 3 đủ A, B, C (T29, 28/10). Còn chữ xám: 2.2.2, 2.2.4, 2.2.5 phần A, C; 2.3.3 phần C; Hình 2.2; review chéo T30, nộp</t>
         </is>
       </c>
     </row>
@@ -5080,7 +5080,7 @@
       </c>
       <c r="G13" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T31: hoàn thiện, nộp báo cáo v2.2 ngày 28/10/2026; Hình 2.2 lược đồ quan hệ; cập nhật kế hoạch
- Báo cáo v2.2: 2.2.2 thêm bước ánh xạ mảng C; 2.2.4 viết lại 19 quan hệ theo A, B, C
  (khóa chính gạch chân) và chèn Hình 2.2; 2.2.5 thêm 12 khóa ngoại C; 2.3.2 thêm 9 quan hệ C,
  2.3.3 chứng minh C, 2.3.4 kết luận A, C; bỏ chữ xám ở 2.2, 2.3, 3; điền ngày nộp.
- docs/3_erd/LuocDo_QuanHe.dot, .png: lược đồ quan hệ vẽ bằng Graphviz, màu theo ERD tổng.
- README: thêm lược đồ quan hệ vào mô tả thư mục 3_erd.
- Kế hoạch: T31 hoàn thành; cập nhật T19, T21, T28, mục 2.2, 2.3 sheet Viết báo cáo;
  báo cáo tuần của Khôi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -1215,7 +1215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="43" min="1" max="2"/>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="L23" s="22" t="inlineStr">
         <is>
-          <t>docs/5_anh-xa/T19_AnhXa_MangA.md – 6 bảng; 8A cho NHAN_VIEN → BAC_SI (partial) và BAC_SI → {ĐA_KHOA, CHUYÊN_KHOA} (disjoint, total), có lý giải (T30 C2 đã chốt); bảng BR-A01…A10 → cơ chế; bảng hành động tham chiếu (T30 L09, 28/10). Báo cáo v2.2 đã có 2.2.3 (lý do 8A); 2.2.5 phần A đã điền (28/10); còn 2.2.2, 2.2.4 phần A, Hình 2.2. Chờ Đăng Khoa review</t>
+          <t>docs/5_anh-xa/T19_AnhXa_MangA.md – 6 bảng; 8A cho NHAN_VIEN → BAC_SI (partial) và BAC_SI → {ĐA_KHOA, CHUYÊN_KHOA} (disjoint, total), có lý giải (T30 C2 đã chốt); bảng BR-A01…A10 → cơ chế; bảng hành động tham chiếu (T30 L09, 28/10). Báo cáo v2.2 đã có 2.2.3 (lý do 8A); 2.2.2, 2.2.4, 2.2.5 phần A, Hình 2.2 đã có trong báo cáo v2.2 (28/10). Chờ Đăng Khoa review</t>
         </is>
       </c>
     </row>
@@ -2473,7 +2473,7 @@
       </c>
       <c r="L25" s="22" t="inlineStr">
         <is>
-          <t>docs/5_anh-xa/T21_AnhXa_MangC.md – 9 bảng; LAN_KHAM.ma_lh UNIQUE NOT NULL (PHÁT_SINH 1:1), không lưu ma_bn/ma_bac_si; 3 bảng kết hợp CHI_TIET_DON_THUOC, THUOC_HOAT_CHAT, DI_UNG; bảng BR-C01…C06 → cơ chế. ten_hoat_chat UNIQUE NOT NULL (T30 L08, 28/10). created_by ánh xạ liên kết GHI_KHÁM, GHI_ĐƠN (T30 C5, ERD C đã vẽ). Báo cáo 2.2 phần C chưa điền. Chờ Khôi review</t>
+          <t>docs/5_anh-xa/T21_AnhXa_MangC.md – 9 bảng; LAN_KHAM.ma_lh UNIQUE NOT NULL (PHÁT_SINH 1:1), không lưu ma_bn/ma_bac_si; 3 bảng kết hợp CHI_TIET_DON_THUOC, THUOC_HOAT_CHAT, DI_UNG; bảng BR-C01…C06 → cơ chế. ten_hoat_chat UNIQUE NOT NULL (T30 L08, 28/10). created_by ánh xạ liên kết GHI_KHÁM, GHI_ĐƠN (T30 C5, ERD C đã vẽ). Báo cáo 2.2 phần C đã điền (T31, 28/10). Chờ Khôi review</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="L32" s="22" t="inlineStr">
         <is>
-          <t>docs/6_chuan-hoa/T28_ChuanHoa_MangC.md – 9 bảng đạt BCNF, không tách (HOAT_CHAT có 2 khóa ứng viên, T30 L08); ghi các dư thừa đã tránh. Báo cáo mục 2.3.3 phần C chưa điền. Chờ Hữu Khoa review</t>
+          <t>docs/6_chuan-hoa/T28_ChuanHoa_MangC.md – 9 bảng đạt BCNF, không tách (HOAT_CHAT có 2 khóa ứng viên, T30 L08); ghi các dư thừa đã tránh. Báo cáo mục 2.3.2–2.3.4 phần C đã điền (T31, 28/10). Chờ Hữu Khoa review</t>
         </is>
       </c>
     </row>
@@ -3025,15 +3025,15 @@
       </c>
       <c r="J35" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="K35" s="21" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="L35" s="22" t="inlineStr">
         <is>
-          <t>docs/INT1313_TX_G5_DeTai05_Telemedicine_v2.2.docx (nháp) – phần B đã điền 2.2, 2.3, 3 (27/10). Phần A đã có 2.2.3 (lý do 8A), 2.3.3. Mục 3 đủ A, B, C (T29, 28/10). 2.2.5 phần A đã điền (28/10). Còn chữ xám: 2.2.2, 2.2.4 phần A, C; 2.2.5 phần C; 2.3.3 phần C; Hình 2.2; nộp (review chéo T30 đã xong 28/10)</t>
+          <t>docs/INT1313_TX_G5_DeTai05_Telemedicine_v2.2.docx – nộp 28/10/2026. Mục 2.2, 2.3, 3 đủ A, B, C: 2.2.2 thêm bước ánh xạ C; 2.2.4 viết lại 19 quan hệ theo A, B, C (khóa chính gạch chân), Hình 2.2 lược đồ quan hệ (docs/3_erd/LuocDo_QuanHe.dot, .png, Graphviz); 2.2.5 thêm 12 khóa ngoại C; 2.3.2 thêm 9 quan hệ C, 2.3.3 chứng minh C, 2.3.4 kết luận A, C; bỏ chữ xám ở 2.2, 2.3, 3; đã review chéo T30</t>
         </is>
       </c>
     </row>
@@ -4345,56 +4345,6 @@
       </c>
       <c r="L59" s="22" t="n"/>
     </row>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
   </sheetData>
   <autoFilter ref="A4:L59"/>
   <conditionalFormatting sqref="A5:E109">
@@ -5010,7 +4960,7 @@
       </c>
       <c r="G11" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -5045,7 +4995,7 @@
       </c>
       <c r="G12" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -5551,24 +5501,21 @@
 T30 (phần B): đối chiếu T20, T24, T27 với DDL, trigger; sửa T20 (FK kép giấy – bệnh nhân); lập danh sách lỗi, bảng quy tắc → cơ chế
 T41 (làm sớm): 4 truy vấn mảng B, kiểm chứng trên dữ liệu thử đi qua trigger
 T31 (nháp v2.2): điền phần B mục 2.2, 2.3, 3 vào báo cáo (đổi tên file sang _v2.2); bổ sung CHECK email, ngày sinh cho benh_nhan theo 1.2.4
-T46 (phần B): điền mục 4.1, 4.2, 5.1 phần B vào báo cáo; T43 (phần B): sql/tests_B.sql 49/49 đạt; Q05–Q08 gói dòng ≤ 80 ký tự, đối chiếu lại khớp</t>
+T46 (phần B): điền mục 4.1, 4.2, 5.1 phần B vào báo cáo; T43 (phần B): sql/tests_B.sql 49/49 đạt; Q05–Q08 gói dòng ≤ 80 ký tự, đối chiếu lại khớp
+28/10: cập nhật kế hoạch mảng A, C; T29: gộp từ điển dữ liệu mục 3 đủ 19 bảng, sửa bảng A lệch cột
+T30: review chéo A, C (chạy trên A_schema chính thức), sửa L07–L14 (SECURITY DEFINER cho trigger, CASCADE mảng A, khóa ứng viên ten_hoat_chat…), chốt C1 (giữ vai_tro, bỏ "đổi vai trò" khỏi BR-B10), C5 (vẽ GHI_KHÁM, GHI_ĐƠN); tests_B 50/50, tests_C 15/15
+T31: hoàn thiện, nộp báo cáo v2.2 (2.2, 2.3 phần C, Hình 2.2 lược đồ quan hệ)</t>
         </is>
       </c>
       <c r="E9" s="22" t="inlineStr">
         <is>
-          <t>T21: review ánh xạ mảng C. T29: điền từ điển dữ liệu bảng mảng B</t>
+          <t>T39: seed A, B (dữ liệu thử T30 làm điểm khởi đầu), gộp seed.sql với Đăng Khoa. T46: điền 4.1–5 phần B, nhắc A, C đưa nội dung vào docx; sửa bảng trigger 4.1.4 còn tên trigger C cũ. T47: khung Flask</t>
         </is>
       </c>
       <c r="F9" s="22" t="inlineStr">
         <is>
-          <t>Hữu Khoa: chốt phương án ánh xạ BAC_SI (8A hay 8C) ở T19 – ảnh hưởng FK ma_bac_si_lap → BAC_SI_DA_KHOA; review T20
-Đăng Khoa: review T24; chốt cách trình bày FD có điều kiện ở T22
-Đăng Khoa: review T27; T30 chốt TAI_KHOAN.vai_tro (giữ hay suy từ loai_nv)
-Hữu Khoa: T18 chốt kiểu khóa (INTEGER identity), giá trị loai_nv trùng vai_tro (QUAN_TRI_NHAN_SU, QUAN_TRI_TAI_KHOAN, QUAN_TRI_DANH_MUC, BAC_SI, LE_TAN); review T33
-Đăng Khoa: review T37; T39 seed phải thêm lịch hẹn ở DA_DAT rồi UPDATE, lịch nằm trong ca, lịch chuyên khoa có giấy hoặc tái khám
-Cả nhóm: họp chốt C1 (TAI_KHOAN.vai_tro trùng loai_nv, BR-B10 đổi vai trò mâu thuẫn BR-A09)
-Hữu Khoa, Đăng Khoa: điền phần A, C vào docs/…_v2.2.docx (chỗ chữ xám); Hữu Khoa vẽ Hình 2.2 lược đồ quan hệ
-Đăng Khoa: gộp tests_B.sql vào tests.sql (T43); T39 seed để có kết quả mẫu Q05–Q08</t>
+          <t>Hữu Khoa: review T29 (6 bảng A viết lại), T30 L09, L10, L13, L14 (đã sửa thay), T35 nối C_schema.sql vào schema.sql
+Đăng Khoa: review T30 L08, L11, L12 (đã sửa thay), ERD C mới (GHI_KHÁM, GHI_ĐƠN); T45 GRANT A, B; đưa nháp T46 phần C vào docx</t>
         </is>
       </c>
       <c r="G9" s="22" t="inlineStr">
@@ -5582,7 +5529,10 @@
 docs/6_chuan-hoa/T30_ReviewCheo.md
 sql/queries_B.sql
 docs/INT1313_TX_G5_DeTai05_Telemedicine_v2.2.docx
-sql/tests_B.sql</t>
+sql/tests_B.sql
+docs/6_chuan-hoa/T30_ReviewCheo.md
+docs/3_erd/C.png, ERD_tong.png, LuocDo_QuanHe.png
+sql/*_trigger_view.sql, tests_B.sql, tests_C.sql</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T35: schema.sql gộp đủ A → B → C, chạy lại từ đầu không lỗi; cập nhật README, kế hoạch
- sql/schema.sql gọi thêm C_schema.sql; chú thích thứ tự phụ thuộc khóa ngoại.
- Chạy lại theo README trên PG16.10: 19 bảng, 6 view, 30 trigger, 25 khóa ngoại; tests_B 50/50.
- README: thêm C_trigger_view.sql vào thứ tự chạy, viết lại ghi chú hợp nhất mảng C.
- Kế hoạch: T35 hoàn thành.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -1215,7 +1215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="43" min="1" max="2"/>
@@ -3249,15 +3249,15 @@
       </c>
       <c r="J39" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="K39" s="21" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="L39" s="22" t="inlineStr">
         <is>
-          <t>sql/schema.sql gọi A_schema → B_schema, chạy được (28/10). Còn nối \ir C_schema.sql (đã thử: A → B → C → A/B/C_trigger_view → rbac chạy liền không lỗi), cập nhật dòng chú thích "C chưa có script"</t>
+          <t>sql/schema.sql gọi A_schema → B_schema → C_schema (28/10, Khôi làm thay Hữu Khoa). Chạy lại từ đầu theo README (createdb → schema → A/B/C_trigger_view → rbac) trên PG16.10 không lỗi: 19 bảng, 6 view, 30 trigger, 25 khóa ngoại; tests_B 50/50. README cập nhật thứ tự chạy (thêm C_trigger_view.sql). Chờ Hữu Khoa review</t>
         </is>
       </c>
     </row>
@@ -4345,6 +4345,56 @@
       </c>
       <c r="L59" s="22" t="n"/>
     </row>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
   </sheetData>
   <autoFilter ref="A4:L59"/>
   <conditionalFormatting sqref="A5:E109">

</xml_diff>

<commit_message>
T43, T45: bộ test phủ đủ 26 BR (124/124 đạt); phân quyền mảng A, B; cập nhật kế hoạch
- tests_A.sql (mới, 35 ca): BR-A01…A10, ràng buộc chung, view; BR-A09 chạy thật dưới từng role.
- tests_B.sql: thêm BR-B08 (6 ca), BR-B10 phân quyền (11 ca); tests_C.sql: thêm 7 ca BR-C06.
  Thủ tục kiểm thử trả role gốc sau mỗi ca.
- tests.sql (mới): gọi tests_A, tests_B, tests_C. Chạy theo README trên PG16.10: A 35, B 67, C 22 đạt.
- rbac.sql: quyền bảng A, B theo BR-A09, B08, B10 và báo cáo 5.2 (quản trị nhân sự không xóa;
  bác sĩ, lễ tân chỉ xem A; lễ tân thêm, sửa bệnh nhân, lịch hẹn; quản trị tài khoản chỉ sửa trang_thai,
  không đọc mật khẩu băm).
- B_trigger_view.sql: view v_lich_hen_cua_toi; hàm tao_tai_khoan_benh_nhan, dat_lai_mat_khau_benh_nhan,
  doi_mat_khau (SECURITY DEFINER, thu hồi EXECUTE của PUBLIC).
- README: ba file test cần rbac.sql. Kế hoạch: cập nhật T43, T45 (80%).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -3313,7 +3313,7 @@
       </c>
       <c r="L40" s="22" t="inlineStr">
         <is>
-          <t>sql/A_trigger_view.sql – 4 constraint trigger trì hoãn trg_phan_lop_* (BR-A01, A02, A10; sửa thứ tự kiểm tra để báo đúng BR-A02, T30 L10); trg_ca_lam_viec_hop_le (BR-A03 giấy phép còn hạn, BR-A08 lịch hẹn không rơi ngoài ca); trg_giay_phep_khong_vo_hieu_ca; trg_ca_lam_viec_khong_xoa (ca có lịch chỉ được HUY); view v_lich_truc_bac_si. Chạy không lỗi (28/10); chưa có test mảng A. Chờ Đăng Khoa review</t>
+          <t>sql/A_trigger_view.sql – 4 constraint trigger trì hoãn trg_phan_lop_* (BR-A01, A02, A10; sửa thứ tự kiểm tra để báo đúng BR-A02, T30 L10); trg_ca_lam_viec_hop_le (BR-A03 giấy phép còn hạn, BR-A08 lịch hẹn không rơi ngoài ca); trg_giay_phep_khong_vo_hieu_ca; trg_ca_lam_viec_khong_xoa (ca có lịch chỉ được HUY); view v_lich_truc_bac_si. Chạy không lỗi (28/10); test ở sql/tests_A.sql 28/28 (T43). Chờ Đăng Khoa review</t>
         </is>
       </c>
     </row>
@@ -3697,15 +3697,15 @@
       </c>
       <c r="J47" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="K47" s="21" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="L47" s="22" t="inlineStr">
         <is>
-          <t>Phần B: sql/tests_B.sql 50/50 trên A_schema chính thức (28/10; sửa dữ liệu A theo A_schema, thêm TB38B theo T30 C1). Phần C: sql/tests_C.sql 15/15 trên A_schema chính thức + dữ liệu thử A, B, gồm TC07A, TC07B chạy dưới role (Khôi, T30, 28/10); chạy lại với seed.sql 15/15 (28/10). Phần A: chưa có test (T30 đã thử tay 13 ca vi phạm, đều bị chặn). Chưa gộp tests.sql</t>
+          <t>sql/tests.sql gọi tests_A.sql (Khôi viết 28/10, 35 ca), tests_B.sql (67 ca), tests_C.sql (22 ca, Đăng Khoa viết, Khôi bổ sung). Phủ đủ 26 BR (A01–A10, B01–B10, C01–C06), kể cả phân quyền BR-A09, B08, B10, C06 bằng ca chạy thật dưới từng role (SET LOCAL ROLE). Chạy theo README (schema → trigger/view → seed → rbac → tests) trên PG16.10 ngày 28/10: 124/124 đạt; tests_A, tests_B cũng đạt khi chưa có seed. Chờ Đăng Khoa review</t>
         </is>
       </c>
     </row>
@@ -3813,11 +3813,11 @@
         </is>
       </c>
       <c r="K49" s="21" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="L49" s="22" t="inlineStr">
         <is>
-          <t>sql/rbac.sql – 6 role NOLOGIN; REVOKE PUBLIC, GRANT phần C (bác sĩ, quản trị danh mục, bệnh nhân chỉ đọc view của mình); A, B mới ghi ma trận ở chú thích. Chạy không lỗi (28/10). Hàm trigger đọc bảng mảng khác đã chuyển SECURITY DEFINER (T30 L11) nên GRANT A, B không cần cấp SELECT chéo mảng. Tên role r_quan_tri_* khác bảng báo cáo 5.2 (r_qt_*) – cần thống nhất. Chờ C1, Khôi review</t>
+          <t>sql/rbac.sql – 6 role NOLOGIN; quyền đủ ba mảng (28/10, Khôi bổ sung A, B): quản trị nhân sự thêm, sửa bảng A, không xóa (BR-A09); bác sĩ, lễ tân chỉ xem A; lễ tân thêm, sửa bệnh nhân, lịch hẹn, không xóa; bác sĩ xem B và lập giấy chuyển (BR-B08); quản trị tài khoản tạo tài khoản, chỉ sửa trang_thai, không đọc mật khẩu băm; lễ tân tạo tài khoản bệnh nhân, đặt lại mật khẩu bệnh nhân qua hàm; mọi người đổi mật khẩu của mình qua doi_mat_khau (BR-B10; hàm, view v_lich_hen_cua_toi ở B_trigger_view.sql); phần C như cũ (BR-C06). Kiểm thử trong tests_A/B/C (T43). Còn: tên role r_quan_tri_* khác bảng báo cáo 5.2 (r_qt_*); Đăng Khoa review, đưa vào báo cáo 5.2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T44: kiểm thử hiệu năng trước/sau chỉ mục trên dữ liệu 1 năm; điền báo cáo 4.2.3; cập nhật kế hoạch
- sql/performance.sql: 6 bài đo PT-01…PT-06 (lịch hôm nay, lịch một bệnh nhân, lịch trực bác sĩ,
  hồ sơ một bệnh nhân, Q09, Q05); "trước chỉ mục" bỏ chỉ mục trong giao dịch rồi ROLLBACK.
  Gộp và thay performance_C.sql.
- seed.sql nhận tham số so_ngay (mặc định 91); đo trên so_ngay=365: 52.437 lịch hẹn, 43.541 lần khám.
  Mã ca dữ liệu mẫu từ 10001 để không đụng dữ liệu thử của tests_A, tests_B.
- Kết quả (trung vị 5 lần, ms): 3,39 → 0,38; 5,37 → 0,04; 0,31 → 0,02; 8,98 → 0,13; 7,99 → 3,41;
  8,06 → 7,63 (tổng hợp toàn bảng, chỉ mục không giúp). Tests 124/124 trên cả dữ liệu 3 tháng và 1 năm.
- Báo cáo 4.2.3: phương pháp đo, bảng kết quả, nhận xét. README: cách chạy đo. Kế hoạch: T44 hoàn thành.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -3753,15 +3753,15 @@
       </c>
       <c r="J48" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="K48" s="21" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="L48" s="22" t="inlineStr">
         <is>
-          <t>sql/performance_C.sql – EXPLAIN (ANALYZE, BUFFERS, VERBOSE) cho lịch sử theo bệnh nhân, tổng hợp thuốc kê, giao hoạt chất – dị ứng; chạy trên fixture nhỏ. Còn: sinh dữ liệu lớn, so sánh trước/sau index, truy vấn A, B</t>
+          <t>sql/performance.sql (Khôi làm 28/10, gộp performance_C.sql của Đăng Khoa): 6 bài đo PT-01…PT-06 trên dữ liệu 1 năm (seed.sql -v so_ngay=365: 52.437 lịch hẹn, 43.541 lần khám, 95 MB); "trước chỉ mục" bỏ chỉ mục trong giao dịch rồi ROLLBACK; trung vị 5 lần. Kết quả (ms, trước → sau): lịch hôm nay 3,39 → 0,38; lịch một bệnh nhân 5,37 → 0,04; lịch trực bác sĩ 0,31 → 0,02; hồ sơ một bệnh nhân 8,98 → 0,13; Q09 7,99 → 3,41; Q05 8,06 → 7,63 (tổng hợp toàn bảng, chỉ mục không giúp). Đã điền báo cáo mục 4.2.3. Chờ Đăng Khoa review</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T45: hoàn thiện báo cáo 5.2 theo rbac.sql; cập nhật 5.1, kế hoạch
- Báo cáo 5.2: bảng quyền 6 role theo đúng tên, quyền trong rbac.sql (thay r_qt_*); nguyên tắc
  đặc quyền tối thiểu; trích lệnh CREATE ROLE/GRANT/REVOKE (khớp rbac.sql); kết quả 31 ca kiểm thử
  phân quyền kèm ví dụ thông báo lỗi; bỏ chữ xám.
- Báo cáo 5.1: mảng B 67 ca (49 từ chối, 17 hợp lệ, 1 view).
- Kế hoạch: T45 hoàn thành; mục 5.2 sheet Viết báo cáo hoàn thành.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -3809,15 +3809,15 @@
       </c>
       <c r="J49" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="K49" s="21" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="L49" s="22" t="inlineStr">
         <is>
-          <t>sql/rbac.sql – 6 role NOLOGIN; quyền đủ ba mảng (28/10, Khôi bổ sung A, B): quản trị nhân sự thêm, sửa bảng A, không xóa (BR-A09); bác sĩ, lễ tân chỉ xem A; lễ tân thêm, sửa bệnh nhân, lịch hẹn, không xóa; bác sĩ xem B và lập giấy chuyển (BR-B08); quản trị tài khoản tạo tài khoản, chỉ sửa trang_thai, không đọc mật khẩu băm; lễ tân tạo tài khoản bệnh nhân, đặt lại mật khẩu bệnh nhân qua hàm; mọi người đổi mật khẩu của mình qua doi_mat_khau (BR-B10; hàm, view v_lich_hen_cua_toi ở B_trigger_view.sql); phần C như cũ (BR-C06). Kiểm thử trong tests_A/B/C (T43). Còn: tên role r_quan_tri_* khác bảng báo cáo 5.2 (r_qt_*); Đăng Khoa review, đưa vào báo cáo 5.2</t>
+          <t>sql/rbac.sql – 6 role NOLOGIN; quyền đủ ba mảng (28/10, Khôi bổ sung A, B): quản trị nhân sự thêm, sửa bảng A, không xóa (BR-A09); bác sĩ, lễ tân chỉ xem A; lễ tân thêm, sửa bệnh nhân, lịch hẹn, không xóa; bác sĩ xem B và lập giấy chuyển (BR-B08); quản trị tài khoản tạo tài khoản, chỉ sửa trang_thai, không đọc mật khẩu băm; lễ tân tạo tài khoản bệnh nhân, đặt lại mật khẩu bệnh nhân qua hàm; mọi người đổi mật khẩu của mình qua doi_mat_khau (BR-B10; hàm, view v_lich_hen_cua_toi ở B_trigger_view.sql); phần C như cũ (BR-C06). Kiểm thử trong tests_A/B/C (T43). Báo cáo 5.2 (28/10): bảng quyền 6 role theo đúng tên, quyền trong rbac.sql (bỏ tên r_qt_* cũ); nguyên tắc đặc quyền tối thiểu, trích lệnh CREATE ROLE/GRANT/REVOKE (đối chiếu khớp rbac.sql); kết quả 31 ca kiểm thử phân quyền kèm ví dụ thông báo lỗi; mục 5.1 cập nhật 67 ca mảng B. Chờ Đăng Khoa review</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5220,7 @@
       </c>
       <c r="G17" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T46: hoàn thiện mục 4, 5 đủ ba mảng; nộp báo cáo v3 ngày 28/10/2026; cập nhật kế hoạch
- Đổi tên báo cáo v2.2 → v3, bìa "Phiên bản: v3 (Cài đặt và truy vấn)".
- Mục 4: môi trường, thứ tự chạy script; 4.1.1 trích DDL mảng A, C; 4.1.2, 4.1.3 chỉ mục, view A, C;
  4.1.4 trigger C đúng tên, ghi chú SECURITY DEFINER; 4.1.5 bảng số bản ghi dữ liệu mẫu;
  4.1.6 cơ chế BR-C01…C06, A09 theo cài đặt; 4.2.1 Q01–Q04, Q09–Q12 theo truy vấn thật;
  4.2.2 thêm Q01–Q04, Q09–Q12 (yêu cầu, SQL, kết quả mẫu, cách hoạt động), điền kết quả mẫu Q05–Q08.
- Mục 5: bỏ chữ xám; 5.1 thêm ca tiêu biểu A, C, tổng kết 124/124.
- queries_A.sql: số hiệu Q01–Q04. Bản nháp T46 phần C ghi đã gộp vào v3.
- Kế hoạch: T46 hoàn thành; mục 4.1, 4.2, 5.1 sheet Viết báo cáo hoàn thành; cập nhật T40, T42.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/KeHoach_G5_Telemedicine.xlsx
+++ b/docs/KeHoach_G5_Telemedicine.xlsx
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L44" s="22" t="inlineStr">
         <is>
-          <t>sql/queries_A.sql – Q1 lịch trực sắp tới + số lịch hẹn trong ca; Q2 bác sĩ có tổng giờ &gt; TB cùng loại; Q3 bác sĩ chưa có ca hiệu lực (NOT EXISTS); Q4 chuyên khoa ≥ 2 bác sĩ có ca trong khoảng tu_luc, den_luc (CTE params, T30 L14). Q2, Q4 khác đề xuất ở sheet Mảng nghiệp vụ (đã cập nhật). Có kết quả trên seed.sql (T39, 28/10). Nên đổi số hiệu Q01–Q04 cho khớp B (Q05–Q08), C (Q09–Q12). Chờ Khôi review</t>
+          <t>sql/queries_A.sql – Q1 lịch trực sắp tới + số lịch hẹn trong ca; Q2 bác sĩ có tổng giờ &gt; TB cùng loại; Q3 bác sĩ chưa có ca hiệu lực (NOT EXISTS); Q4 chuyên khoa ≥ 2 bác sĩ có ca trong khoảng tu_luc, den_luc (CTE params, T30 L14). Q2, Q4 khác đề xuất ở sheet Mảng nghiệp vụ (đã cập nhật). Có kết quả trên seed.sql (T39, 28/10). Chờ Khôi review. Đã trình bày ở báo cáo v3 mục 4.2.2 kèm kết quả mẫu (T46).</t>
         </is>
       </c>
     </row>
@@ -3649,7 +3649,7 @@
       </c>
       <c r="L46" s="22" t="inlineStr">
         <is>
-          <t>sql/queries_C.sql – Q09 top 10 thuốc theo quý; Q10 bệnh nhân có mã ICD chưa tái khám sau 30 ngày; Q11 lịch sử lâm sàng 1 bệnh nhân (JOIN 5+ bảng); Q12 bác sĩ có số thuốc TB/đơn &gt; mức chung; tham số trong CTE params. Chạy được; có kết quả trên fixture của Đăng Khoa, có kết quả trên seed.sql (T39, 28/10). Chờ Hữu Khoa review</t>
+          <t>sql/queries_C.sql – Q09 top 10 thuốc theo quý; Q10 bệnh nhân có mã ICD chưa tái khám sau 30 ngày; Q11 lịch sử lâm sàng 1 bệnh nhân (JOIN 5+ bảng); Q12 bác sĩ có số thuốc TB/đơn &gt; mức chung; tham số trong CTE params. Chạy được; có kết quả trên fixture của Đăng Khoa, có kết quả trên seed.sql (T39, 28/10). Chờ Hữu Khoa review. Đã trình bày ở báo cáo v3 mục 4.2.2 kèm kết quả mẫu (T46).</t>
         </is>
       </c>
     </row>
@@ -3865,15 +3865,15 @@
       </c>
       <c r="J50" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="K50" s="21" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="L50" s="22" t="inlineStr">
         <is>
-          <t>Phần B đã vào docs/…_v2.2.docx (27/10). Phần C: nháp docs/7_bao-cao/T46_DuThao_Muc_4_1_4_2_5.md (4.1.6, 4.2, 5), chưa vào docx. Phần A: chưa có (4.1 DDL, view, trigger từ T32, T36; 4.2 Q1–Q4). Chờ seed T39 (kết quả mẫu), T44 số đo, T45 GRANT A, B; nộp v3</t>
+          <t>docs/INT1313_TX_G5_DeTai05_Telemedicine_v3.docx – nộp 28/10/2026 (đổi tên từ v2.2, bìa "Phiên bản: v3"). Mục 4: môi trường, thứ tự chạy script; 4.1.1 thêm A (ca_lam_viec), C (lan_kham, chi_tiet_don_thuoc); 4.1.2 chỉ mục A, C; 4.1.3 view C, v_lich_hen_cua_toi; 4.1.4 trigger C đúng tên (thay 3 dòng tên cũ), ghi chú SECURITY DEFINER; 4.1.5 bảng số bản ghi seed 3 tháng; 4.1.6 cơ chế C, A09 theo cài đặt; 4.2.1 Q01–Q04, Q09–Q12 theo truy vấn thật; 4.2.2 thêm A, C (yêu cầu, SQL, kết quả mẫu từ seed, cách hoạt động), điền kết quả mẫu Q05–Q08; 4.2.3 (T44). Mục 5: 5.1 thêm ca tiêu biểu A, C (35 dòng), tổng kết 124/124; 5.2 (T45). Bỏ hết chữ xám mục 4, 5; queries_A.sql đổi số hiệu Q01–Q04</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
       </c>
       <c r="G14" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -5150,7 +5150,7 @@
       </c>
       <c r="G15" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5185,7 @@
       </c>
       <c r="G16" s="20" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>